<commit_message>
Added four test scenarios in Po with free of cost and fixed random failures
Added four test scenarios in Po with free of cost and fixed random failures
</commit_message>
<xml_diff>
--- a/testdata/Purchase-FOC Scenarios.xlsx
+++ b/testdata/Purchase-FOC Scenarios.xlsx
@@ -9,13 +9,15 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6915" firstSheet="2" activeTab="3"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6915" firstSheet="1" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="DomesticPoFOCUDGeneralSameUOM" sheetId="11" r:id="rId1"/>
-    <sheet name="DomesticPoFOCUDServiceSameUOM" sheetId="21" r:id="rId2"/>
-    <sheet name="ImportPoFOCUDGeneralSameUOM" sheetId="17" r:id="rId3"/>
-    <sheet name="ImportPoFOCUDServiceSameUOM" sheetId="13" r:id="rId4"/>
+    <sheet name="DomesticPoFOCUDGeneralDiffUOM" sheetId="22" r:id="rId2"/>
+    <sheet name="ImportPoFOCUDGeneralDiffUOM" sheetId="23" r:id="rId3"/>
+    <sheet name="DomesticPoFOCUDServiceSameUOM" sheetId="21" r:id="rId4"/>
+    <sheet name="ImportPoFOCUDGeneralSameUOM" sheetId="17" r:id="rId5"/>
+    <sheet name="ImportPoFOCUDServiceSameUOM" sheetId="13" r:id="rId6"/>
   </sheets>
   <calcPr calcId="152511"/>
   <extLst>
@@ -35,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="572" uniqueCount="105">
   <si>
     <t>Purchase Order &amp; GRN</t>
   </si>
@@ -301,6 +303,12 @@
     <t>Total</t>
   </si>
   <si>
+    <t>GWL_ITEM_DISSIMILAR_UOM</t>
+  </si>
+  <si>
+    <t>KGS</t>
+  </si>
+  <si>
     <t>GWL_Item_FP_service_01</t>
   </si>
   <si>
@@ -341,6 +349,9 @@
   </si>
   <si>
     <t>RM WH-49</t>
+  </si>
+  <si>
+    <t>GWL_ITEM_DISSIMILAR_UOM_DESC</t>
   </si>
 </sst>
 </file>
@@ -415,7 +426,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79976805932798245"/>
+        <fgColor theme="7" tint="0.79973754081850645"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -445,7 +456,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79973754081850645"/>
+        <fgColor theme="7" tint="0.79970702230903046"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1463,7 +1474,7 @@
       </c>
       <c r="AC4" s="8">
         <f>IF($V2=1,S4+AB4,S4)</f>
-        <v>734.81000000000006</v>
+        <v>734.81</v>
       </c>
       <c r="AD4" s="8">
         <v>120</v>
@@ -1641,7 +1652,7 @@
       </c>
       <c r="AC5" s="25">
         <f t="shared" si="1"/>
-        <v>734.81000000000006</v>
+        <v>734.81</v>
       </c>
       <c r="AD5" s="26">
         <f t="shared" si="1"/>
@@ -1805,7 +1816,7 @@
       </c>
       <c r="B2" s="51"/>
       <c r="C2" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>2</v>
@@ -2111,13 +2122,13 @@
         <v>88</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>88</v>
+        <v>104</v>
       </c>
       <c r="D4" s="7" t="s">
         <v>76</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>76</v>
+        <v>89</v>
       </c>
       <c r="F4" s="8">
         <v>5</v>
@@ -2178,15 +2189,15 @@
       </c>
       <c r="V4" s="8">
         <f>IF(OR($C$2=1,$C$2=4),ROUND((((S4*U4)/100)/2),2),0)</f>
-        <v>0</v>
+        <v>56.04</v>
       </c>
       <c r="W4" s="8">
         <f>IF($C$2=1,ROUND((((S4*U4)/100)/2),2),0)</f>
-        <v>0</v>
+        <v>56.04</v>
       </c>
       <c r="X4" s="8">
         <f>IF($C$2=2,ROUND(((S4*U4)/100),2),0)</f>
-        <v>112.09</v>
+        <v>0</v>
       </c>
       <c r="Y4" s="8">
         <f>IF($C$2=4,ROUND((((S4*U4)/100)/2),2),0)</f>
@@ -2196,15 +2207,16 @@
         <v>0</v>
       </c>
       <c r="AA4" s="8">
+        <f>IF($C2=3,0,(S4*Z4)/100)</f>
         <v>0</v>
       </c>
       <c r="AB4" s="8">
         <f>V4+W4+X4+Y4+AA4</f>
-        <v>112.09</v>
+        <v>112.08</v>
       </c>
       <c r="AC4" s="8">
         <f>IF($V2=1,S4+AB4,S4)</f>
-        <v>734.81000000000006</v>
+        <v>734.80000000000007</v>
       </c>
       <c r="AD4" s="8">
         <v>120</v>
@@ -2363,26 +2375,26 @@
       <c r="U5" s="20"/>
       <c r="V5" s="21">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>56.04</v>
       </c>
       <c r="W5" s="21">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>56.04</v>
       </c>
       <c r="X5" s="21">
         <f t="shared" si="0"/>
-        <v>112.09</v>
+        <v>0</v>
       </c>
       <c r="Y5" s="21"/>
       <c r="Z5" s="21"/>
       <c r="AA5" s="21"/>
       <c r="AB5" s="20">
         <f t="shared" ref="AB5:AE5" si="1">SUM(AB4:AB4)</f>
-        <v>112.09</v>
+        <v>112.08</v>
       </c>
       <c r="AC5" s="25">
         <f t="shared" si="1"/>
-        <v>734.81000000000006</v>
+        <v>734.80000000000007</v>
       </c>
       <c r="AD5" s="26">
         <f t="shared" si="1"/>
@@ -2849,16 +2861,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>75</v>
+        <v>104</v>
       </c>
       <c r="D4" s="7" t="s">
         <v>76</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>76</v>
+        <v>89</v>
       </c>
       <c r="F4" s="8">
         <v>5</v>
@@ -2934,7 +2946,7 @@
         <v>0</v>
       </c>
       <c r="Z4" s="8">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AA4" s="8">
         <f>IF($C2=3,0,(S4*Z4)/100)</f>
@@ -2977,15 +2989,15 @@
         <v>0</v>
       </c>
       <c r="AL4" s="8">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AM4" s="8">
         <f>F4/AL4</f>
-        <v>1.6666666666666701</v>
+        <v>5</v>
       </c>
       <c r="AN4" s="8">
         <f>AI4/AM4</f>
-        <v>373.63200000000001</v>
+        <v>124.544</v>
       </c>
       <c r="AO4" s="8">
         <f>AJ4/AM4</f>
@@ -3000,7 +3012,7 @@
       </c>
       <c r="AR4" s="33">
         <f>ROUND(AN4+AO4+AP4,5)</f>
-        <v>373.63200000000001</v>
+        <v>124.544</v>
       </c>
       <c r="AS4" s="33" t="s">
         <v>77</v>
@@ -3016,19 +3028,19 @@
       </c>
       <c r="AW4" s="32">
         <f>AM4</f>
-        <v>1.6666666666666701</v>
+        <v>5</v>
       </c>
       <c r="AX4" s="32">
         <f>AR4</f>
-        <v>373.63200000000001</v>
+        <v>124.544</v>
       </c>
       <c r="AY4" s="32">
         <f>AU4+AW4</f>
-        <v>14091.666666666701</v>
+        <v>14095</v>
       </c>
       <c r="AZ4" s="32">
         <f>ROUND(((AU4*AV4)+(AW4*AX4))/(AU4+AW4),5)</f>
-        <v>121.25023</v>
+        <v>121.22156</v>
       </c>
       <c r="BA4" s="36"/>
       <c r="BB4" s="36" t="s">
@@ -3060,11 +3072,11 @@
       </c>
       <c r="BO4" s="32">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
-        <v>146.79804999999999</v>
+        <v>146.67549</v>
       </c>
       <c r="BP4" s="40">
         <f>BN4+AW4</f>
-        <v>692.66666666666697</v>
+        <v>696</v>
       </c>
       <c r="BQ4" s="41">
         <v>123562</v>
@@ -3197,6 +3209,1489 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:BQ5"/>
+  <sheetFormatPr defaultColWidth="9.85546875" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="9.85546875" style="1"/>
+    <col min="2" max="2" width="25.5703125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="26" style="1" customWidth="1"/>
+    <col min="4" max="19" width="9.85546875" style="1"/>
+    <col min="20" max="20" width="10.140625" style="1" customWidth="1"/>
+    <col min="21" max="16384" width="9.85546875" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:69">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
+      <c r="K1" s="15"/>
+      <c r="L1" s="15"/>
+      <c r="M1" s="15"/>
+      <c r="N1" s="15"/>
+      <c r="O1" s="15"/>
+      <c r="P1" s="15"/>
+      <c r="Q1" s="15"/>
+      <c r="R1" s="2"/>
+      <c r="S1" s="2"/>
+      <c r="T1" s="2"/>
+      <c r="U1" s="2"/>
+      <c r="V1" s="2"/>
+      <c r="W1" s="2"/>
+      <c r="X1" s="2"/>
+      <c r="Y1" s="2"/>
+      <c r="Z1" s="2"/>
+      <c r="AA1" s="2"/>
+      <c r="AB1" s="2"/>
+      <c r="AC1" s="2"/>
+      <c r="AD1" s="2"/>
+      <c r="AE1" s="2"/>
+      <c r="AF1" s="2"/>
+      <c r="AG1" s="2"/>
+      <c r="AH1" s="2"/>
+      <c r="AI1" s="2"/>
+      <c r="AJ1" s="2"/>
+      <c r="AK1" s="2"/>
+      <c r="AL1" s="2"/>
+      <c r="AM1" s="2"/>
+      <c r="AN1" s="2"/>
+      <c r="AO1" s="2"/>
+      <c r="AP1" s="2"/>
+      <c r="AQ1" s="2"/>
+      <c r="AR1" s="2"/>
+      <c r="AS1" s="10"/>
+      <c r="AT1" s="33"/>
+      <c r="AU1" s="33"/>
+      <c r="AV1" s="33"/>
+      <c r="AW1" s="33"/>
+      <c r="AX1" s="33"/>
+      <c r="AY1" s="33"/>
+      <c r="AZ1" s="33"/>
+      <c r="BA1" s="33"/>
+      <c r="BB1" s="33"/>
+      <c r="BC1" s="33"/>
+      <c r="BD1" s="33"/>
+      <c r="BE1" s="33"/>
+      <c r="BF1" s="33"/>
+      <c r="BG1" s="33"/>
+      <c r="BH1" s="33"/>
+      <c r="BI1" s="33"/>
+      <c r="BJ1" s="33"/>
+      <c r="BK1" s="33"/>
+      <c r="BL1" s="33"/>
+      <c r="BM1" s="33"/>
+      <c r="BN1" s="33"/>
+      <c r="BO1" s="33"/>
+      <c r="BP1" s="33"/>
+      <c r="BQ1" s="33"/>
+    </row>
+    <row r="2" spans="1:69">
+      <c r="A2" s="51" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="51"/>
+      <c r="C2" s="4">
+        <v>2</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="J2" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="K2" s="15"/>
+      <c r="L2" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="M2" s="15">
+        <v>1</v>
+      </c>
+      <c r="N2" s="15"/>
+      <c r="O2" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="P2" s="15">
+        <v>1</v>
+      </c>
+      <c r="Q2" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="R2" s="2"/>
+      <c r="S2" s="2"/>
+      <c r="T2" s="2"/>
+      <c r="U2" s="2"/>
+      <c r="V2" s="2">
+        <v>1</v>
+      </c>
+      <c r="W2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="X2" s="2"/>
+      <c r="Y2" s="2"/>
+      <c r="Z2" s="2"/>
+      <c r="AA2" s="2"/>
+      <c r="AB2" s="2"/>
+      <c r="AC2" s="2"/>
+      <c r="AD2" s="2"/>
+      <c r="AE2" s="2"/>
+      <c r="AF2" s="2"/>
+      <c r="AG2" s="2"/>
+      <c r="AH2" s="2"/>
+      <c r="AI2" s="2"/>
+      <c r="AJ2" s="2"/>
+      <c r="AK2" s="2"/>
+      <c r="AL2" s="2"/>
+      <c r="AM2" s="2"/>
+      <c r="AN2" s="2"/>
+      <c r="AO2" s="2"/>
+      <c r="AP2" s="2"/>
+      <c r="AQ2" s="2"/>
+      <c r="AR2" s="2"/>
+      <c r="AS2" s="10"/>
+      <c r="AT2" s="33"/>
+      <c r="AU2" s="33"/>
+      <c r="AV2" s="33"/>
+      <c r="AW2" s="33"/>
+      <c r="AX2" s="33"/>
+      <c r="AY2" s="33"/>
+      <c r="AZ2" s="33"/>
+      <c r="BA2" s="33"/>
+      <c r="BB2" s="33"/>
+      <c r="BC2" s="33"/>
+      <c r="BD2" s="33"/>
+      <c r="BE2" s="33"/>
+      <c r="BF2" s="33"/>
+      <c r="BG2" s="33"/>
+      <c r="BH2" s="33"/>
+      <c r="BI2" s="33"/>
+      <c r="BJ2" s="33"/>
+      <c r="BK2" s="33"/>
+      <c r="BL2" s="33"/>
+      <c r="BM2" s="33"/>
+      <c r="BN2" s="33"/>
+      <c r="BO2" s="33"/>
+      <c r="BP2" s="33"/>
+      <c r="BQ2" s="33"/>
+    </row>
+    <row r="3" spans="1:69" ht="60">
+      <c r="A3" s="42" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="42" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="43" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="42" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="42" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="44" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" s="42" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" s="42" t="s">
+        <v>16</v>
+      </c>
+      <c r="I3" s="45" t="s">
+        <v>17</v>
+      </c>
+      <c r="J3" s="45" t="s">
+        <v>18</v>
+      </c>
+      <c r="K3" s="45" t="s">
+        <v>19</v>
+      </c>
+      <c r="L3" s="46" t="s">
+        <v>20</v>
+      </c>
+      <c r="M3" s="46" t="s">
+        <v>21</v>
+      </c>
+      <c r="N3" s="46" t="s">
+        <v>22</v>
+      </c>
+      <c r="O3" s="46" t="s">
+        <v>23</v>
+      </c>
+      <c r="P3" s="46" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q3" s="46" t="s">
+        <v>25</v>
+      </c>
+      <c r="R3" s="45" t="s">
+        <v>26</v>
+      </c>
+      <c r="S3" s="42" t="s">
+        <v>27</v>
+      </c>
+      <c r="T3" s="42" t="s">
+        <v>28</v>
+      </c>
+      <c r="U3" s="22" t="s">
+        <v>29</v>
+      </c>
+      <c r="V3" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="W3" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="X3" s="22" t="s">
+        <v>32</v>
+      </c>
+      <c r="Y3" s="22" t="s">
+        <v>33</v>
+      </c>
+      <c r="Z3" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="AA3" s="22" t="s">
+        <v>35</v>
+      </c>
+      <c r="AB3" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="AC3" s="47" t="s">
+        <v>37</v>
+      </c>
+      <c r="AD3" s="47" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE3" s="48" t="s">
+        <v>39</v>
+      </c>
+      <c r="AF3" s="48" t="s">
+        <v>40</v>
+      </c>
+      <c r="AG3" s="48" t="s">
+        <v>41</v>
+      </c>
+      <c r="AH3" s="47" t="s">
+        <v>42</v>
+      </c>
+      <c r="AI3" s="47" t="s">
+        <v>43</v>
+      </c>
+      <c r="AJ3" s="48" t="s">
+        <v>44</v>
+      </c>
+      <c r="AK3" s="48" t="s">
+        <v>45</v>
+      </c>
+      <c r="AL3" s="47" t="s">
+        <v>46</v>
+      </c>
+      <c r="AM3" s="47" t="s">
+        <v>47</v>
+      </c>
+      <c r="AN3" s="48" t="s">
+        <v>48</v>
+      </c>
+      <c r="AO3" s="48" t="s">
+        <v>49</v>
+      </c>
+      <c r="AP3" s="48" t="s">
+        <v>50</v>
+      </c>
+      <c r="AQ3" s="47" t="s">
+        <v>51</v>
+      </c>
+      <c r="AR3" s="49" t="s">
+        <v>52</v>
+      </c>
+      <c r="AS3" s="29" t="s">
+        <v>53</v>
+      </c>
+      <c r="AT3" s="29" t="s">
+        <v>51</v>
+      </c>
+      <c r="AU3" s="30" t="s">
+        <v>54</v>
+      </c>
+      <c r="AV3" s="30" t="s">
+        <v>55</v>
+      </c>
+      <c r="AW3" s="30" t="s">
+        <v>56</v>
+      </c>
+      <c r="AX3" s="30" t="s">
+        <v>57</v>
+      </c>
+      <c r="AY3" s="30" t="s">
+        <v>58</v>
+      </c>
+      <c r="AZ3" s="30" t="s">
+        <v>59</v>
+      </c>
+      <c r="BA3" s="30" t="s">
+        <v>60</v>
+      </c>
+      <c r="BB3" s="30" t="s">
+        <v>61</v>
+      </c>
+      <c r="BC3" s="34" t="s">
+        <v>62</v>
+      </c>
+      <c r="BD3" s="34" t="s">
+        <v>63</v>
+      </c>
+      <c r="BE3" s="34" t="s">
+        <v>64</v>
+      </c>
+      <c r="BF3" s="30" t="s">
+        <v>65</v>
+      </c>
+      <c r="BG3" s="30" t="s">
+        <v>66</v>
+      </c>
+      <c r="BH3" s="30" t="s">
+        <v>67</v>
+      </c>
+      <c r="BI3" s="30" t="s">
+        <v>68</v>
+      </c>
+      <c r="BJ3" s="30" t="s">
+        <v>69</v>
+      </c>
+      <c r="BK3" s="30" t="s">
+        <v>70</v>
+      </c>
+      <c r="BL3" s="30" t="s">
+        <v>71</v>
+      </c>
+      <c r="BM3" s="30" t="s">
+        <v>72</v>
+      </c>
+      <c r="BN3" s="30" t="s">
+        <v>73</v>
+      </c>
+      <c r="BO3" s="30" t="s">
+        <v>59</v>
+      </c>
+      <c r="BP3" s="30" t="s">
+        <v>74</v>
+      </c>
+      <c r="BQ3" s="30" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:69">
+      <c r="A4" s="7">
+        <v>1</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="F4" s="8">
+        <v>5</v>
+      </c>
+      <c r="G4" s="8">
+        <v>150</v>
+      </c>
+      <c r="H4" s="8">
+        <f>F4*G4</f>
+        <v>750</v>
+      </c>
+      <c r="I4" s="8">
+        <v>5</v>
+      </c>
+      <c r="J4" s="8">
+        <v>8</v>
+      </c>
+      <c r="K4" s="8">
+        <v>5</v>
+      </c>
+      <c r="L4" s="8">
+        <f>H4</f>
+        <v>750</v>
+      </c>
+      <c r="M4" s="8">
+        <f>ROUND(L4*I4%,2)</f>
+        <v>37.5</v>
+      </c>
+      <c r="N4" s="8">
+        <f>H4-M4</f>
+        <v>712.5</v>
+      </c>
+      <c r="O4" s="8">
+        <f>ROUND(N4*J4%,2)</f>
+        <v>57</v>
+      </c>
+      <c r="P4" s="8">
+        <f>ROUND(N4-O4,2)</f>
+        <v>655.5</v>
+      </c>
+      <c r="Q4" s="8">
+        <f>ROUND(P4*K4%,2)</f>
+        <v>32.78</v>
+      </c>
+      <c r="R4" s="8">
+        <f>M4+O4+Q4</f>
+        <v>127.28</v>
+      </c>
+      <c r="S4" s="8">
+        <f>(H4-R4)</f>
+        <v>622.72</v>
+      </c>
+      <c r="T4" s="8">
+        <v>88363222</v>
+      </c>
+      <c r="U4" s="8">
+        <v>18</v>
+      </c>
+      <c r="V4" s="8">
+        <f>IF(OR($C$2=1,$C$2=4),ROUND((((S4*U4)/100)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="W4" s="8">
+        <f>IF($C$2=1,ROUND((((S4*U4)/100)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="X4" s="8">
+        <f>IF($C$2=2,ROUND(((S4*U4)/100),2),0)</f>
+        <v>112.09</v>
+      </c>
+      <c r="Y4" s="8">
+        <f>IF($C$2=4,ROUND((((S4*U4)/100)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Z4" s="8">
+        <v>0</v>
+      </c>
+      <c r="AA4" s="8">
+        <v>0</v>
+      </c>
+      <c r="AB4" s="8">
+        <f>V4+W4+X4+Y4+AA4</f>
+        <v>112.09</v>
+      </c>
+      <c r="AC4" s="8">
+        <f>IF($V2=1,S4+AB4,S4)</f>
+        <v>734.81</v>
+      </c>
+      <c r="AD4" s="8">
+        <v>120</v>
+      </c>
+      <c r="AE4" s="8">
+        <f>IF($P$2=1,(S4/$S$5)*$E$16,AD4/$AD$5*$E$16)</f>
+        <v>0</v>
+      </c>
+      <c r="AF4" s="8"/>
+      <c r="AG4" s="8">
+        <f>IF($P$2=1,(S4/$S$5)*$E$18,AD4/$AD$5*$E$18)</f>
+        <v>0</v>
+      </c>
+      <c r="AH4" s="8">
+        <f>IF($P$2=1,(S4/$S$5)*$E$18,AD4/$AD$5*$E$18)</f>
+        <v>0</v>
+      </c>
+      <c r="AI4" s="8">
+        <f>S4*$M$2</f>
+        <v>622.72</v>
+      </c>
+      <c r="AJ4" s="8">
+        <f>IF($C$2=3,0,AG4+AH4)</f>
+        <v>0</v>
+      </c>
+      <c r="AK4" s="8">
+        <f>IF($C$2=3,AE4+AG4+AH4,0)</f>
+        <v>0</v>
+      </c>
+      <c r="AL4" s="8">
+        <v>1</v>
+      </c>
+      <c r="AM4" s="8">
+        <f>F4/AL4</f>
+        <v>5</v>
+      </c>
+      <c r="AN4" s="8">
+        <f>AI4/AM4</f>
+        <v>124.544</v>
+      </c>
+      <c r="AO4" s="8">
+        <f>AJ4/AM4</f>
+        <v>0</v>
+      </c>
+      <c r="AP4" s="8">
+        <f>AK4/AM4</f>
+        <v>0</v>
+      </c>
+      <c r="AQ4" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="AR4" s="33">
+        <f>ROUND(AN4+AO4+AP4,5)</f>
+        <v>124.544</v>
+      </c>
+      <c r="AS4" s="33" t="s">
+        <v>77</v>
+      </c>
+      <c r="AT4" s="32" t="s">
+        <v>76</v>
+      </c>
+      <c r="AU4" s="33" t="s">
+        <v>78</v>
+      </c>
+      <c r="AV4" s="33" t="s">
+        <v>79</v>
+      </c>
+      <c r="AW4" s="32">
+        <f>AM4</f>
+        <v>5</v>
+      </c>
+      <c r="AX4" s="32">
+        <f>AR4</f>
+        <v>124.544</v>
+      </c>
+      <c r="AY4" s="32">
+        <f>AU4+AW4</f>
+        <v>14095</v>
+      </c>
+      <c r="AZ4" s="32">
+        <f>ROUND(((AU4*AV4)+(AW4*AX4))/(AU4+AW4),5)</f>
+        <v>121.22156</v>
+      </c>
+      <c r="BA4" s="36"/>
+      <c r="BB4" s="36" t="s">
+        <v>80</v>
+      </c>
+      <c r="BC4" s="50" t="s">
+        <v>81</v>
+      </c>
+      <c r="BD4" s="38" t="s">
+        <v>82</v>
+      </c>
+      <c r="BE4" s="38" t="s">
+        <v>83</v>
+      </c>
+      <c r="BF4" s="36"/>
+      <c r="BG4" s="36"/>
+      <c r="BH4" s="36"/>
+      <c r="BI4" s="32"/>
+      <c r="BJ4" s="33"/>
+      <c r="BK4" s="33"/>
+      <c r="BL4" s="32" t="s">
+        <v>84</v>
+      </c>
+      <c r="BM4" s="33" t="s">
+        <v>85</v>
+      </c>
+      <c r="BN4" s="33" t="s">
+        <v>86</v>
+      </c>
+      <c r="BO4" s="32">
+        <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
+        <v>146.67549</v>
+      </c>
+      <c r="BP4" s="40">
+        <f>BN4+AW4</f>
+        <v>696</v>
+      </c>
+      <c r="BQ4" s="41">
+        <v>123562</v>
+      </c>
+    </row>
+    <row r="5" spans="1:69">
+      <c r="A5" s="10"/>
+      <c r="B5" s="11"/>
+      <c r="C5" s="11"/>
+      <c r="D5" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="E5" s="12"/>
+      <c r="F5" s="12"/>
+      <c r="G5" s="13"/>
+      <c r="H5" s="14">
+        <f>SUM(H4:H4)</f>
+        <v>750</v>
+      </c>
+      <c r="I5" s="7"/>
+      <c r="J5" s="7"/>
+      <c r="K5" s="7"/>
+      <c r="L5" s="7"/>
+      <c r="M5" s="7"/>
+      <c r="N5" s="7"/>
+      <c r="O5" s="7"/>
+      <c r="P5" s="7"/>
+      <c r="Q5" s="7"/>
+      <c r="R5" s="20">
+        <f t="shared" ref="R5:X5" si="0">SUM(R4:R4)</f>
+        <v>127.28</v>
+      </c>
+      <c r="S5" s="14">
+        <f t="shared" si="0"/>
+        <v>622.72</v>
+      </c>
+      <c r="T5" s="20"/>
+      <c r="U5" s="20"/>
+      <c r="V5" s="21">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="W5" s="21">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="X5" s="21">
+        <f t="shared" si="0"/>
+        <v>112.09</v>
+      </c>
+      <c r="Y5" s="21"/>
+      <c r="Z5" s="21"/>
+      <c r="AA5" s="21"/>
+      <c r="AB5" s="20">
+        <f t="shared" ref="AB5:AE5" si="1">SUM(AB4:AB4)</f>
+        <v>112.09</v>
+      </c>
+      <c r="AC5" s="25">
+        <f t="shared" si="1"/>
+        <v>734.81</v>
+      </c>
+      <c r="AD5" s="26">
+        <f t="shared" si="1"/>
+        <v>120</v>
+      </c>
+      <c r="AE5" s="26">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AF5" s="25"/>
+      <c r="AG5" s="26">
+        <f t="shared" ref="AG5:AK5" si="2">SUM(AG4:AG4)</f>
+        <v>0</v>
+      </c>
+      <c r="AH5" s="26">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AI5" s="26">
+        <f t="shared" si="2"/>
+        <v>622.72</v>
+      </c>
+      <c r="AJ5" s="26">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AK5" s="26">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AL5" s="25"/>
+      <c r="AM5" s="25"/>
+      <c r="AN5" s="25"/>
+      <c r="AO5" s="25"/>
+      <c r="AP5" s="25"/>
+      <c r="AQ5" s="25"/>
+      <c r="AR5" s="25"/>
+      <c r="AS5" s="10"/>
+      <c r="AT5" s="33"/>
+      <c r="AU5" s="33"/>
+      <c r="AV5" s="33"/>
+      <c r="AW5" s="33"/>
+      <c r="AX5" s="33"/>
+      <c r="AY5" s="33"/>
+      <c r="AZ5" s="33"/>
+      <c r="BA5" s="33"/>
+      <c r="BB5" s="33"/>
+      <c r="BC5" s="33"/>
+      <c r="BD5" s="33"/>
+      <c r="BE5" s="33"/>
+      <c r="BF5" s="33"/>
+      <c r="BG5" s="33"/>
+      <c r="BH5" s="33"/>
+      <c r="BI5" s="33"/>
+      <c r="BJ5" s="33"/>
+      <c r="BK5" s="33"/>
+      <c r="BL5" s="33"/>
+      <c r="BM5" s="33"/>
+      <c r="BN5" s="33"/>
+      <c r="BO5" s="33"/>
+      <c r="BP5" s="33"/>
+      <c r="BQ5" s="33"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:B2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:BQ5"/>
+  <sheetFormatPr defaultColWidth="9.85546875" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="9.85546875" style="1"/>
+    <col min="2" max="2" width="25.5703125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="26" style="1" customWidth="1"/>
+    <col min="4" max="19" width="9.85546875" style="1"/>
+    <col min="20" max="20" width="10.140625" style="1" customWidth="1"/>
+    <col min="21" max="16384" width="9.85546875" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:69">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
+      <c r="K1" s="15"/>
+      <c r="L1" s="15"/>
+      <c r="M1" s="15"/>
+      <c r="N1" s="15"/>
+      <c r="O1" s="15"/>
+      <c r="P1" s="15"/>
+      <c r="Q1" s="15"/>
+      <c r="R1" s="2"/>
+      <c r="S1" s="2"/>
+      <c r="T1" s="2"/>
+      <c r="U1" s="2"/>
+      <c r="V1" s="2"/>
+      <c r="W1" s="2"/>
+      <c r="X1" s="2"/>
+      <c r="Y1" s="2"/>
+      <c r="Z1" s="2"/>
+      <c r="AA1" s="2"/>
+      <c r="AB1" s="2"/>
+      <c r="AC1" s="2"/>
+      <c r="AD1" s="2"/>
+      <c r="AE1" s="2"/>
+      <c r="AF1" s="2"/>
+      <c r="AG1" s="2"/>
+      <c r="AH1" s="2"/>
+      <c r="AI1" s="2"/>
+      <c r="AJ1" s="2"/>
+      <c r="AK1" s="2"/>
+      <c r="AL1" s="2"/>
+      <c r="AM1" s="2"/>
+      <c r="AN1" s="2"/>
+      <c r="AO1" s="2"/>
+      <c r="AP1" s="2"/>
+      <c r="AQ1" s="2"/>
+      <c r="AR1" s="2"/>
+      <c r="AS1" s="10"/>
+      <c r="AT1" s="33"/>
+      <c r="AU1" s="33"/>
+      <c r="AV1" s="33"/>
+      <c r="AW1" s="33"/>
+      <c r="AX1" s="33"/>
+      <c r="AY1" s="33"/>
+      <c r="AZ1" s="33"/>
+      <c r="BA1" s="33"/>
+      <c r="BB1" s="33"/>
+      <c r="BC1" s="33"/>
+      <c r="BD1" s="33"/>
+      <c r="BE1" s="33"/>
+      <c r="BF1" s="33"/>
+      <c r="BG1" s="33"/>
+      <c r="BH1" s="33"/>
+      <c r="BI1" s="33"/>
+      <c r="BJ1" s="33"/>
+      <c r="BK1" s="33"/>
+      <c r="BL1" s="33"/>
+      <c r="BM1" s="33"/>
+      <c r="BN1" s="33"/>
+      <c r="BO1" s="33"/>
+      <c r="BP1" s="33"/>
+      <c r="BQ1" s="33"/>
+    </row>
+    <row r="2" spans="1:69">
+      <c r="A2" s="51" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="51"/>
+      <c r="C2" s="4">
+        <v>3</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="J2" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="K2" s="15"/>
+      <c r="L2" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="M2" s="15">
+        <v>1</v>
+      </c>
+      <c r="N2" s="15"/>
+      <c r="O2" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="P2" s="15">
+        <v>1</v>
+      </c>
+      <c r="Q2" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="R2" s="2"/>
+      <c r="S2" s="2"/>
+      <c r="T2" s="2"/>
+      <c r="U2" s="2"/>
+      <c r="V2" s="2">
+        <v>1</v>
+      </c>
+      <c r="W2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="X2" s="2"/>
+      <c r="Y2" s="2"/>
+      <c r="Z2" s="2"/>
+      <c r="AA2" s="2"/>
+      <c r="AB2" s="2"/>
+      <c r="AC2" s="2"/>
+      <c r="AD2" s="2"/>
+      <c r="AE2" s="2"/>
+      <c r="AF2" s="2"/>
+      <c r="AG2" s="2"/>
+      <c r="AH2" s="2"/>
+      <c r="AI2" s="2"/>
+      <c r="AJ2" s="2"/>
+      <c r="AK2" s="2"/>
+      <c r="AL2" s="2"/>
+      <c r="AM2" s="2"/>
+      <c r="AN2" s="2"/>
+      <c r="AO2" s="2"/>
+      <c r="AP2" s="2"/>
+      <c r="AQ2" s="2"/>
+      <c r="AR2" s="2"/>
+      <c r="AS2" s="10"/>
+      <c r="AT2" s="33"/>
+      <c r="AU2" s="33"/>
+      <c r="AV2" s="33"/>
+      <c r="AW2" s="33"/>
+      <c r="AX2" s="33"/>
+      <c r="AY2" s="33"/>
+      <c r="AZ2" s="33"/>
+      <c r="BA2" s="33"/>
+      <c r="BB2" s="33"/>
+      <c r="BC2" s="33"/>
+      <c r="BD2" s="33"/>
+      <c r="BE2" s="33"/>
+      <c r="BF2" s="33"/>
+      <c r="BG2" s="33"/>
+      <c r="BH2" s="33"/>
+      <c r="BI2" s="33"/>
+      <c r="BJ2" s="33"/>
+      <c r="BK2" s="33"/>
+      <c r="BL2" s="33"/>
+      <c r="BM2" s="33"/>
+      <c r="BN2" s="33"/>
+      <c r="BO2" s="33"/>
+      <c r="BP2" s="33"/>
+      <c r="BQ2" s="33"/>
+    </row>
+    <row r="3" spans="1:69" ht="60">
+      <c r="A3" s="42" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="42" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="43" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="42" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="42" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="44" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" s="42" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" s="42" t="s">
+        <v>16</v>
+      </c>
+      <c r="I3" s="45" t="s">
+        <v>17</v>
+      </c>
+      <c r="J3" s="45" t="s">
+        <v>18</v>
+      </c>
+      <c r="K3" s="45" t="s">
+        <v>19</v>
+      </c>
+      <c r="L3" s="46" t="s">
+        <v>20</v>
+      </c>
+      <c r="M3" s="46" t="s">
+        <v>21</v>
+      </c>
+      <c r="N3" s="46" t="s">
+        <v>22</v>
+      </c>
+      <c r="O3" s="46" t="s">
+        <v>23</v>
+      </c>
+      <c r="P3" s="46" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q3" s="46" t="s">
+        <v>25</v>
+      </c>
+      <c r="R3" s="45" t="s">
+        <v>26</v>
+      </c>
+      <c r="S3" s="42" t="s">
+        <v>27</v>
+      </c>
+      <c r="T3" s="42" t="s">
+        <v>28</v>
+      </c>
+      <c r="U3" s="22" t="s">
+        <v>29</v>
+      </c>
+      <c r="V3" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="W3" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="X3" s="22" t="s">
+        <v>32</v>
+      </c>
+      <c r="Y3" s="22" t="s">
+        <v>33</v>
+      </c>
+      <c r="Z3" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="AA3" s="22" t="s">
+        <v>35</v>
+      </c>
+      <c r="AB3" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="AC3" s="47" t="s">
+        <v>37</v>
+      </c>
+      <c r="AD3" s="47" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE3" s="48" t="s">
+        <v>39</v>
+      </c>
+      <c r="AF3" s="48" t="s">
+        <v>40</v>
+      </c>
+      <c r="AG3" s="48" t="s">
+        <v>41</v>
+      </c>
+      <c r="AH3" s="47" t="s">
+        <v>42</v>
+      </c>
+      <c r="AI3" s="47" t="s">
+        <v>43</v>
+      </c>
+      <c r="AJ3" s="48" t="s">
+        <v>44</v>
+      </c>
+      <c r="AK3" s="48" t="s">
+        <v>45</v>
+      </c>
+      <c r="AL3" s="47" t="s">
+        <v>46</v>
+      </c>
+      <c r="AM3" s="47" t="s">
+        <v>47</v>
+      </c>
+      <c r="AN3" s="48" t="s">
+        <v>48</v>
+      </c>
+      <c r="AO3" s="48" t="s">
+        <v>49</v>
+      </c>
+      <c r="AP3" s="48" t="s">
+        <v>50</v>
+      </c>
+      <c r="AQ3" s="47" t="s">
+        <v>51</v>
+      </c>
+      <c r="AR3" s="49" t="s">
+        <v>52</v>
+      </c>
+      <c r="AS3" s="29" t="s">
+        <v>53</v>
+      </c>
+      <c r="AT3" s="29" t="s">
+        <v>51</v>
+      </c>
+      <c r="AU3" s="30" t="s">
+        <v>54</v>
+      </c>
+      <c r="AV3" s="30" t="s">
+        <v>55</v>
+      </c>
+      <c r="AW3" s="30" t="s">
+        <v>56</v>
+      </c>
+      <c r="AX3" s="30" t="s">
+        <v>57</v>
+      </c>
+      <c r="AY3" s="30" t="s">
+        <v>58</v>
+      </c>
+      <c r="AZ3" s="30" t="s">
+        <v>59</v>
+      </c>
+      <c r="BA3" s="30" t="s">
+        <v>60</v>
+      </c>
+      <c r="BB3" s="30" t="s">
+        <v>61</v>
+      </c>
+      <c r="BC3" s="34" t="s">
+        <v>62</v>
+      </c>
+      <c r="BD3" s="34" t="s">
+        <v>63</v>
+      </c>
+      <c r="BE3" s="34" t="s">
+        <v>64</v>
+      </c>
+      <c r="BF3" s="30" t="s">
+        <v>65</v>
+      </c>
+      <c r="BG3" s="30" t="s">
+        <v>66</v>
+      </c>
+      <c r="BH3" s="30" t="s">
+        <v>67</v>
+      </c>
+      <c r="BI3" s="30" t="s">
+        <v>68</v>
+      </c>
+      <c r="BJ3" s="30" t="s">
+        <v>69</v>
+      </c>
+      <c r="BK3" s="30" t="s">
+        <v>70</v>
+      </c>
+      <c r="BL3" s="30" t="s">
+        <v>71</v>
+      </c>
+      <c r="BM3" s="30" t="s">
+        <v>72</v>
+      </c>
+      <c r="BN3" s="30" t="s">
+        <v>73</v>
+      </c>
+      <c r="BO3" s="30" t="s">
+        <v>59</v>
+      </c>
+      <c r="BP3" s="30" t="s">
+        <v>74</v>
+      </c>
+      <c r="BQ3" s="30" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:69">
+      <c r="A4" s="7">
+        <v>1</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="F4" s="8">
+        <v>5</v>
+      </c>
+      <c r="G4" s="8">
+        <v>150</v>
+      </c>
+      <c r="H4" s="8">
+        <f>F4*G4</f>
+        <v>750</v>
+      </c>
+      <c r="I4" s="8">
+        <v>5</v>
+      </c>
+      <c r="J4" s="8">
+        <v>8</v>
+      </c>
+      <c r="K4" s="8">
+        <v>5</v>
+      </c>
+      <c r="L4" s="8">
+        <f>H4</f>
+        <v>750</v>
+      </c>
+      <c r="M4" s="8">
+        <f>ROUND(L4*I4%,2)</f>
+        <v>37.5</v>
+      </c>
+      <c r="N4" s="8">
+        <f>H4-M4</f>
+        <v>712.5</v>
+      </c>
+      <c r="O4" s="8">
+        <f>ROUND(N4*J4%,2)</f>
+        <v>57</v>
+      </c>
+      <c r="P4" s="8">
+        <f>ROUND(N4-O4,2)</f>
+        <v>655.5</v>
+      </c>
+      <c r="Q4" s="8">
+        <f>ROUND(P4*K4%,2)</f>
+        <v>32.78</v>
+      </c>
+      <c r="R4" s="8">
+        <f>M4+O4+Q4</f>
+        <v>127.28</v>
+      </c>
+      <c r="S4" s="8">
+        <f>(H4-R4)</f>
+        <v>622.72</v>
+      </c>
+      <c r="T4" s="8">
+        <v>88363222</v>
+      </c>
+      <c r="U4" s="8">
+        <v>0</v>
+      </c>
+      <c r="V4" s="8">
+        <f>IF(OR($C$2=1,$C$2=4),ROUND((((S4*U4)/100)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="W4" s="8">
+        <f>IF($C$2=1,ROUND((((S4*U4)/100)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="X4" s="8">
+        <f>IF($C$2=2,ROUND(((S4*U4)/100),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Y4" s="8">
+        <f>IF($C$2=4,ROUND((((S4*U4)/100)/2),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Z4" s="8">
+        <v>4</v>
+      </c>
+      <c r="AA4" s="8">
+        <f>IF($C2=3,0,(S4*Z4)/100)</f>
+        <v>0</v>
+      </c>
+      <c r="AB4" s="8">
+        <f>V4+W4+X4+Y4+AA4</f>
+        <v>0</v>
+      </c>
+      <c r="AC4" s="8">
+        <f>IF($V2=1,S4+AB4,S4)</f>
+        <v>622.72</v>
+      </c>
+      <c r="AD4" s="8">
+        <v>120</v>
+      </c>
+      <c r="AE4" s="8">
+        <f>IF($P$2=1,(S4/$S$5)*$E$16,AD4/$AD$5*$E$16)</f>
+        <v>0</v>
+      </c>
+      <c r="AF4" s="8"/>
+      <c r="AG4" s="8">
+        <f>IF($P$2=1,(S4/$S$5)*$E$18,AD4/$AD$5*$E$18)</f>
+        <v>0</v>
+      </c>
+      <c r="AH4" s="8">
+        <f>IF($P$2=1,(S4/$S$5)*$E$18,AD4/$AD$5*$E$18)</f>
+        <v>0</v>
+      </c>
+      <c r="AI4" s="8">
+        <f>S4*$M$2</f>
+        <v>622.72</v>
+      </c>
+      <c r="AJ4" s="8">
+        <f>IF($C$2=3,0,AG4+AH4)</f>
+        <v>0</v>
+      </c>
+      <c r="AK4" s="8">
+        <f>IF($C$2=3,AE4+AG4+AH4,0)</f>
+        <v>0</v>
+      </c>
+      <c r="AL4" s="8">
+        <v>3</v>
+      </c>
+      <c r="AM4" s="8">
+        <f>F4/AL4</f>
+        <v>1.6666666666666701</v>
+      </c>
+      <c r="AN4" s="8">
+        <f>AI4/AM4</f>
+        <v>373.63200000000001</v>
+      </c>
+      <c r="AO4" s="8">
+        <f>AJ4/AM4</f>
+        <v>0</v>
+      </c>
+      <c r="AP4" s="8">
+        <f>AK4/AM4</f>
+        <v>0</v>
+      </c>
+      <c r="AQ4" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="AR4" s="33">
+        <f>ROUND(AN4+AO4+AP4,5)</f>
+        <v>373.63200000000001</v>
+      </c>
+      <c r="AS4" s="33" t="s">
+        <v>77</v>
+      </c>
+      <c r="AT4" s="32" t="s">
+        <v>76</v>
+      </c>
+      <c r="AU4" s="33" t="s">
+        <v>78</v>
+      </c>
+      <c r="AV4" s="33" t="s">
+        <v>79</v>
+      </c>
+      <c r="AW4" s="32">
+        <f>AM4</f>
+        <v>1.6666666666666701</v>
+      </c>
+      <c r="AX4" s="32">
+        <f>AR4</f>
+        <v>373.63200000000001</v>
+      </c>
+      <c r="AY4" s="32">
+        <f>AU4+AW4</f>
+        <v>14091.666666666701</v>
+      </c>
+      <c r="AZ4" s="32">
+        <f>ROUND(((AU4*AV4)+(AW4*AX4))/(AU4+AW4),5)</f>
+        <v>121.25023</v>
+      </c>
+      <c r="BA4" s="36"/>
+      <c r="BB4" s="36" t="s">
+        <v>80</v>
+      </c>
+      <c r="BC4" s="50" t="s">
+        <v>81</v>
+      </c>
+      <c r="BD4" s="38" t="s">
+        <v>82</v>
+      </c>
+      <c r="BE4" s="38" t="s">
+        <v>83</v>
+      </c>
+      <c r="BF4" s="36"/>
+      <c r="BG4" s="36"/>
+      <c r="BH4" s="36"/>
+      <c r="BI4" s="32"/>
+      <c r="BJ4" s="33"/>
+      <c r="BK4" s="33"/>
+      <c r="BL4" s="32" t="s">
+        <v>84</v>
+      </c>
+      <c r="BM4" s="33" t="s">
+        <v>85</v>
+      </c>
+      <c r="BN4" s="33" t="s">
+        <v>86</v>
+      </c>
+      <c r="BO4" s="32">
+        <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
+        <v>146.79804999999999</v>
+      </c>
+      <c r="BP4" s="40">
+        <f>BN4+AW4</f>
+        <v>692.66666666666697</v>
+      </c>
+      <c r="BQ4" s="41">
+        <v>123562</v>
+      </c>
+    </row>
+    <row r="5" spans="1:69">
+      <c r="A5" s="10"/>
+      <c r="B5" s="11"/>
+      <c r="C5" s="11"/>
+      <c r="D5" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="E5" s="12"/>
+      <c r="F5" s="12"/>
+      <c r="G5" s="13"/>
+      <c r="H5" s="14">
+        <f>SUM(H4:H4)</f>
+        <v>750</v>
+      </c>
+      <c r="I5" s="7"/>
+      <c r="J5" s="7"/>
+      <c r="K5" s="7"/>
+      <c r="L5" s="7"/>
+      <c r="M5" s="7"/>
+      <c r="N5" s="7"/>
+      <c r="O5" s="7"/>
+      <c r="P5" s="7"/>
+      <c r="Q5" s="7"/>
+      <c r="R5" s="20">
+        <f t="shared" ref="R5:X5" si="0">SUM(R4:R4)</f>
+        <v>127.28</v>
+      </c>
+      <c r="S5" s="14">
+        <f t="shared" si="0"/>
+        <v>622.72</v>
+      </c>
+      <c r="T5" s="20"/>
+      <c r="U5" s="20"/>
+      <c r="V5" s="21">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="W5" s="21">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="X5" s="21">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="Y5" s="21"/>
+      <c r="Z5" s="21"/>
+      <c r="AA5" s="21"/>
+      <c r="AB5" s="20">
+        <f t="shared" ref="AB5:AE5" si="1">SUM(AB4:AB4)</f>
+        <v>0</v>
+      </c>
+      <c r="AC5" s="25">
+        <f t="shared" si="1"/>
+        <v>622.72</v>
+      </c>
+      <c r="AD5" s="26">
+        <f t="shared" si="1"/>
+        <v>120</v>
+      </c>
+      <c r="AE5" s="26">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AF5" s="25"/>
+      <c r="AG5" s="26">
+        <f t="shared" ref="AG5:AK5" si="2">SUM(AG4:AG4)</f>
+        <v>0</v>
+      </c>
+      <c r="AH5" s="26">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AI5" s="26">
+        <f t="shared" si="2"/>
+        <v>622.72</v>
+      </c>
+      <c r="AJ5" s="26">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AK5" s="26">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AL5" s="25"/>
+      <c r="AM5" s="25"/>
+      <c r="AN5" s="25"/>
+      <c r="AO5" s="25"/>
+      <c r="AP5" s="25"/>
+      <c r="AQ5" s="25"/>
+      <c r="AR5" s="25"/>
+      <c r="AS5" s="10"/>
+      <c r="AT5" s="33"/>
+      <c r="AU5" s="33"/>
+      <c r="AV5" s="33"/>
+      <c r="AW5" s="33"/>
+      <c r="AX5" s="33"/>
+      <c r="AY5" s="33"/>
+      <c r="AZ5" s="33"/>
+      <c r="BA5" s="33"/>
+      <c r="BB5" s="33"/>
+      <c r="BC5" s="33"/>
+      <c r="BD5" s="33"/>
+      <c r="BE5" s="33"/>
+      <c r="BF5" s="33"/>
+      <c r="BG5" s="33"/>
+      <c r="BH5" s="33"/>
+      <c r="BI5" s="33"/>
+      <c r="BJ5" s="33"/>
+      <c r="BK5" s="33"/>
+      <c r="BL5" s="33"/>
+      <c r="BM5" s="33"/>
+      <c r="BN5" s="33"/>
+      <c r="BO5" s="33"/>
+      <c r="BP5" s="33"/>
+      <c r="BQ5" s="33"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:B2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
@@ -3379,13 +4874,13 @@
     </row>
     <row r="3" spans="1:69" ht="60">
       <c r="A3" s="6" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B3" s="6" t="s">
         <v>10</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D3" s="6" t="s">
         <v>12</v>
@@ -3394,7 +4889,7 @@
         <v>13</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="G3" s="6" t="s">
         <v>15</v>
@@ -3424,7 +4919,7 @@
         <v>25</v>
       </c>
       <c r="P3" s="17" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="Q3" s="17" t="s">
         <v>23</v>
@@ -3433,13 +4928,13 @@
         <v>26</v>
       </c>
       <c r="S3" s="6" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="T3" s="6" t="s">
         <v>28</v>
       </c>
       <c r="U3" s="18" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="V3" s="18" t="s">
         <v>30</v>
@@ -3508,7 +5003,7 @@
         <v>51</v>
       </c>
       <c r="AR3" s="28" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="AS3" s="29" t="s">
         <v>53</v>
@@ -3591,10 +5086,10 @@
         <v>1</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D4" s="7" t="s">
         <v>76</v>
@@ -3606,14 +5101,14 @@
         <v>5</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="H4" s="8">
         <f>F4*G4</f>
         <v>250</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="J4" s="8">
         <v>8</v>
@@ -3745,16 +5240,16 @@
         <v>41.514000000000003</v>
       </c>
       <c r="AS4" s="31" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="AT4" s="32" t="s">
         <v>76</v>
       </c>
       <c r="AU4" s="9" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="AV4" s="9" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="AW4" s="32">
         <f>AM4</f>
@@ -3792,13 +5287,13 @@
       <c r="BJ4" s="32"/>
       <c r="BK4" s="32"/>
       <c r="BL4" s="39" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="BM4" s="9" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="BN4" s="9" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="BO4" s="32">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>

</xml_diff>

<commit_message>
Added stock calculation test scripts and FOC test scenarios
Added stock calculation test scripts and FOC test scenarios
</commit_message>
<xml_diff>
--- a/testdata/Purchase-FOC Scenarios.xlsx
+++ b/testdata/Purchase-FOC Scenarios.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="6920" firstSheet="16" activeTab="17"/>
+    <workbookView windowWidth="19200" windowHeight="6200" firstSheet="24" activeTab="25"/>
   </bookViews>
   <sheets>
     <sheet name="DomesticPoFOCUDGeneralSameUOM" sheetId="11" r:id="rId1"/>
@@ -27,22 +27,26 @@
     <sheet name="D-PoToGRNFOCPLStkTrnSameUOMWI" sheetId="53" r:id="rId18"/>
     <sheet name="D-PoToGRNFOCRCStkTrnSameUOMWI" sheetId="51" r:id="rId19"/>
     <sheet name="D-PoToGRNFOCUDStkTrnDiffUOMWOI" sheetId="48" r:id="rId20"/>
-    <sheet name="D-PoToGRNFOCUDStkTrnSameUOMWI" sheetId="47" r:id="rId21"/>
-    <sheet name="D-PoToGRNFOCUDStkTrnDiffUOMWI" sheetId="49" r:id="rId22"/>
-    <sheet name="D-PoToGRNFOCUDServiceSameUOMWOI" sheetId="42" r:id="rId23"/>
-    <sheet name="D-PoToGRNFOCRCGeneralSameUOMWOI" sheetId="34" r:id="rId24"/>
-    <sheet name="D-PoToGRNFOCRCServiceSameUOMWOI" sheetId="43" r:id="rId25"/>
-    <sheet name="D-PoToGRNFOCPLGeneralSameUOMWOI" sheetId="37" r:id="rId26"/>
-    <sheet name="D-PoToGRNFOCPLServiceSameUOMWOI" sheetId="44" r:id="rId27"/>
-    <sheet name="D-PoToGRNFOCUDGeneralDiffUOMWOI" sheetId="31" r:id="rId28"/>
-    <sheet name="D-PoToGRNFOCRCGeneralDiffUOMWOI" sheetId="38" r:id="rId29"/>
-    <sheet name="D-PoToGRNFOCPLGeneralDiffUOMWOI" sheetId="41" r:id="rId30"/>
-    <sheet name="D-PoToGRNFOCUDGeneralSameUOMWI" sheetId="32" r:id="rId31"/>
-    <sheet name="D-PoToGRNFOCRCGeneralSameUOMWI" sheetId="35" r:id="rId32"/>
-    <sheet name="D-PoToGRNFOCPLGeneralSameUOMWI" sheetId="36" r:id="rId33"/>
-    <sheet name="D-PoToGRNFOCUDGeneralDiffUOMWI" sheetId="33" r:id="rId34"/>
-    <sheet name="D-PoToGRNFOCRCGeneralDiffUOMWI" sheetId="39" r:id="rId35"/>
-    <sheet name="D-PoToGRNFOCPLGeneralDiffUOMWI" sheetId="40" r:id="rId36"/>
+    <sheet name="D-PoToGRNFOCRCStkTrnDiffUOMWOI" sheetId="54" r:id="rId21"/>
+    <sheet name="D-PoToGRNFOCPLStkTrnDiffUOMWOI" sheetId="55" r:id="rId22"/>
+    <sheet name="D-PoToGRNFOCUDStkTrnSameUOMWI" sheetId="47" r:id="rId23"/>
+    <sheet name="D-PoToGRNFOCUDStkTrnDiffUOMWI" sheetId="49" r:id="rId24"/>
+    <sheet name="D-PoToGRNFOCRCStkTrnDiffUOMWI" sheetId="57" r:id="rId25"/>
+    <sheet name="D-PoToGRNFOCPLStkTrnDiffUOMWI" sheetId="58" r:id="rId26"/>
+    <sheet name="D-PoToGRNFOCUDServiceSameUOMWOI" sheetId="42" r:id="rId27"/>
+    <sheet name="D-PoToGRNFOCRCGeneralSameUOMWOI" sheetId="34" r:id="rId28"/>
+    <sheet name="D-PoToGRNFOCRCServiceSameUOMWOI" sheetId="43" r:id="rId29"/>
+    <sheet name="D-PoToGRNFOCPLGeneralSameUOMWOI" sheetId="37" r:id="rId30"/>
+    <sheet name="D-PoToGRNFOCPLServiceSameUOMWOI" sheetId="44" r:id="rId31"/>
+    <sheet name="D-PoToGRNFOCUDGeneralDiffUOMWOI" sheetId="31" r:id="rId32"/>
+    <sheet name="D-PoToGRNFOCRCGeneralDiffUOMWOI" sheetId="38" r:id="rId33"/>
+    <sheet name="D-PoToGRNFOCPLGeneralDiffUOMWOI" sheetId="41" r:id="rId34"/>
+    <sheet name="D-PoToGRNFOCUDGeneralSameUOMWI" sheetId="32" r:id="rId35"/>
+    <sheet name="D-PoToGRNFOCRCGeneralSameUOMWI" sheetId="35" r:id="rId36"/>
+    <sheet name="D-PoToGRNFOCPLGeneralSameUOMWI" sheetId="36" r:id="rId37"/>
+    <sheet name="D-PoToGRNFOCUDGeneralDiffUOMWI" sheetId="33" r:id="rId38"/>
+    <sheet name="D-PoToGRNFOCRCGeneralDiffUOMWI" sheetId="39" r:id="rId39"/>
+    <sheet name="D-PoToGRNFOCPLGeneralDiffUOMWI" sheetId="40" r:id="rId40"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -62,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3302" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3682" uniqueCount="139">
   <si>
     <t>Purchase Order &amp; GRN</t>
   </si>
@@ -430,10 +434,22 @@
     <t>GWL_Dissimilar_St_02</t>
   </si>
   <si>
+    <t>GWL_Item_Dissimilar_Rc_02</t>
+  </si>
+  <si>
+    <t>GWL_Item_Dissimilar_Pl_03</t>
+  </si>
+  <si>
     <t>GWL_Item_Similar_St_08</t>
   </si>
   <si>
     <t>GWL_Dissimilar_St_01</t>
+  </si>
+  <si>
+    <t>GWL_Item_Dissimilar_Rc_01</t>
+  </si>
+  <si>
+    <t>GWL_Item_Dissimilar_Pl_01</t>
   </si>
   <si>
     <t>GWL_Item_service_05</t>
@@ -454,9 +470,6 @@
     <t>GWL_Item_Dissimilar_05</t>
   </si>
   <si>
-    <t>GWL_Item_Dissimilar_Rc_02</t>
-  </si>
-  <si>
     <t>GWL_Item_Dissimilar_Pl_02</t>
   </si>
   <si>
@@ -470,12 +483,6 @@
   </si>
   <si>
     <t>GWL_Item_Dissimilar_04</t>
-  </si>
-  <si>
-    <t>GWL_Item_Dissimilar_Rc_01</t>
-  </si>
-  <si>
-    <t>GWL_Item_Dissimilar_Pl_01</t>
   </si>
 </sst>
 </file>
@@ -10554,7 +10561,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:69">
+    <row r="4" ht="15.25" spans="1:69">
       <c r="A4" s="77">
         <v>1</v>
       </c>
@@ -16592,6 +16599,10 @@
   <sheetPr/>
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5" outlineLevelRow="4"/>
+  <cols>
+    <col min="2" max="2" width="21.5454545454545" customWidth="1"/>
+    <col min="3" max="3" width="27.8181818181818" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:69">
       <c r="A1" s="1" t="s">
@@ -17187,7 +17198,7 @@
       <c r="P5" s="7"/>
       <c r="Q5" s="7"/>
       <c r="R5" s="13">
-        <f t="shared" ref="R5:AK5" si="0">SUM(R4:R4)</f>
+        <f t="shared" ref="R5:X5" si="0">SUM(R4:R4)</f>
         <v>71.53</v>
       </c>
       <c r="S5" s="13">
@@ -17208,56 +17219,44 @@
         <f t="shared" si="0"/>
         <v>59.12</v>
       </c>
-      <c r="Y5" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="Z5" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="AA5" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
+      <c r="Y5" s="38"/>
+      <c r="Z5" s="38"/>
+      <c r="AA5" s="38"/>
       <c r="AB5" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="AB5:AE5" si="1">SUM(AB4:AB4)</f>
         <v>59.12</v>
       </c>
       <c r="AC5" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>328.47</v>
       </c>
       <c r="AD5" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>120</v>
       </c>
       <c r="AE5" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="AF5" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AF5" s="23"/>
       <c r="AG5" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="AG5:AK5" si="2">SUM(AG4:AG4)</f>
         <v>0</v>
       </c>
       <c r="AH5" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AI5" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>328.47</v>
       </c>
       <c r="AJ5" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AK5" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AL5" s="23"/>
@@ -17310,6 +17309,10 @@
   <sheetPr/>
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5" outlineLevelRow="4"/>
+  <cols>
+    <col min="2" max="2" width="21.5454545454545" customWidth="1"/>
+    <col min="3" max="3" width="27.8181818181818" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:69">
       <c r="A1" s="1" t="s">
@@ -17905,7 +17908,7 @@
       <c r="P5" s="7"/>
       <c r="Q5" s="7"/>
       <c r="R5" s="13">
-        <f t="shared" ref="R5:AK5" si="0">SUM(R4:R4)</f>
+        <f t="shared" ref="R5:X5" si="0">SUM(R4:R4)</f>
         <v>71.53</v>
       </c>
       <c r="S5" s="13">
@@ -17926,56 +17929,44 @@
         <f t="shared" si="0"/>
         <v>59.12</v>
       </c>
-      <c r="Y5" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="Z5" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="AA5" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
+      <c r="Y5" s="38"/>
+      <c r="Z5" s="38"/>
+      <c r="AA5" s="38"/>
       <c r="AB5" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="AB5:AE5" si="1">SUM(AB4:AB4)</f>
         <v>59.12</v>
       </c>
       <c r="AC5" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>328.47</v>
       </c>
       <c r="AD5" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>120</v>
       </c>
       <c r="AE5" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="AF5" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AF5" s="23"/>
       <c r="AG5" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="AG5:AK5" si="2">SUM(AG4:AG4)</f>
         <v>0</v>
       </c>
       <c r="AH5" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AI5" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>328.47</v>
       </c>
       <c r="AJ5" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AK5" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AL5" s="23"/>
@@ -18772,6 +18763,10 @@
   <sheetPr/>
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5" outlineLevelRow="4"/>
+  <cols>
+    <col min="2" max="2" width="21.5454545454545" customWidth="1"/>
+    <col min="3" max="3" width="27.8181818181818" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:69">
       <c r="A1" s="1" t="s">
@@ -19367,7 +19362,7 @@
       <c r="P5" s="7"/>
       <c r="Q5" s="7"/>
       <c r="R5" s="13">
-        <f t="shared" ref="R5:AK5" si="0">SUM(R4:R4)</f>
+        <f t="shared" ref="R5:X5" si="0">SUM(R4:R4)</f>
         <v>71.53</v>
       </c>
       <c r="S5" s="13">
@@ -19388,56 +19383,44 @@
         <f t="shared" si="0"/>
         <v>59.12</v>
       </c>
-      <c r="Y5" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="Z5" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="AA5" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
+      <c r="Y5" s="38"/>
+      <c r="Z5" s="38"/>
+      <c r="AA5" s="38"/>
       <c r="AB5" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="AB5:AE5" si="1">SUM(AB4:AB4)</f>
         <v>59.12</v>
       </c>
       <c r="AC5" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>328.47</v>
       </c>
       <c r="AD5" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>120</v>
       </c>
       <c r="AE5" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="AF5" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AF5" s="23"/>
       <c r="AG5" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="AG5:AK5" si="2">SUM(AG4:AG4)</f>
         <v>0</v>
       </c>
       <c r="AH5" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AI5" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>328.47</v>
       </c>
       <c r="AJ5" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AK5" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AL5" s="23"/>
@@ -19490,6 +19473,10 @@
   <sheetPr/>
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5" outlineLevelRow="4"/>
+  <cols>
+    <col min="2" max="2" width="21.5454545454545" customWidth="1"/>
+    <col min="3" max="3" width="27.8181818181818" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:69">
       <c r="A1" s="1" t="s">
@@ -20085,7 +20072,7 @@
       <c r="P5" s="7"/>
       <c r="Q5" s="7"/>
       <c r="R5" s="13">
-        <f t="shared" ref="R5:AK5" si="0">SUM(R4:R4)</f>
+        <f t="shared" ref="R5:X5" si="0">SUM(R4:R4)</f>
         <v>71.53</v>
       </c>
       <c r="S5" s="13">
@@ -20106,56 +20093,44 @@
         <f t="shared" si="0"/>
         <v>59.12</v>
       </c>
-      <c r="Y5" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="Z5" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="AA5" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
+      <c r="Y5" s="38"/>
+      <c r="Z5" s="38"/>
+      <c r="AA5" s="38"/>
       <c r="AB5" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="AB5:AE5" si="1">SUM(AB4:AB4)</f>
         <v>59.12</v>
       </c>
       <c r="AC5" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>328.47</v>
       </c>
       <c r="AD5" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>120</v>
       </c>
       <c r="AE5" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="AF5" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AF5" s="23"/>
       <c r="AG5" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="AG5:AK5" si="2">SUM(AG4:AG4)</f>
         <v>0</v>
       </c>
       <c r="AH5" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AI5" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>328.47</v>
       </c>
       <c r="AJ5" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AK5" s="13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AL5" s="23"/>
@@ -21309,10 +21284,10 @@
         <v>1</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>134</v>
+        <v>122</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>134</v>
+        <v>122</v>
       </c>
       <c r="D4" s="7" t="s">
         <v>76</v>
@@ -22027,10 +22002,10 @@
         <v>1</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D4" s="7" t="s">
         <v>76</v>
@@ -22745,10 +22720,10 @@
         <v>1</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D4" s="7" t="s">
         <v>76</v>
@@ -23463,10 +23438,2168 @@
         <v>1</v>
       </c>
       <c r="B4" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="F4" s="8">
+        <v>4</v>
+      </c>
+      <c r="G4" s="8">
+        <v>100</v>
+      </c>
+      <c r="H4" s="8">
+        <v>400</v>
+      </c>
+      <c r="I4" s="8">
+        <v>4</v>
+      </c>
+      <c r="J4" s="8">
+        <v>9</v>
+      </c>
+      <c r="K4" s="8">
+        <v>6</v>
+      </c>
+      <c r="L4" s="8">
+        <v>400</v>
+      </c>
+      <c r="M4" s="8">
+        <v>16</v>
+      </c>
+      <c r="N4" s="8">
+        <v>384</v>
+      </c>
+      <c r="O4" s="8">
+        <v>34.56</v>
+      </c>
+      <c r="P4" s="8">
+        <v>349.44</v>
+      </c>
+      <c r="Q4" s="8">
+        <v>20.97</v>
+      </c>
+      <c r="R4" s="8">
+        <v>71.53</v>
+      </c>
+      <c r="S4" s="8">
+        <v>328.47</v>
+      </c>
+      <c r="T4" s="8">
+        <v>88363222</v>
+      </c>
+      <c r="U4" s="8">
+        <v>18</v>
+      </c>
+      <c r="V4" s="8">
+        <v>0</v>
+      </c>
+      <c r="W4" s="8">
+        <v>0</v>
+      </c>
+      <c r="X4" s="8">
+        <v>59.12</v>
+      </c>
+      <c r="Y4" s="8">
+        <v>0</v>
+      </c>
+      <c r="Z4" s="8">
+        <v>0</v>
+      </c>
+      <c r="AA4" s="8">
+        <v>0</v>
+      </c>
+      <c r="AB4" s="8">
+        <v>59.12</v>
+      </c>
+      <c r="AC4" s="8">
+        <v>328.47</v>
+      </c>
+      <c r="AD4" s="21">
+        <v>120</v>
+      </c>
+      <c r="AE4" s="21">
+        <v>0</v>
+      </c>
+      <c r="AF4" s="21"/>
+      <c r="AG4" s="21">
+        <v>0</v>
+      </c>
+      <c r="AH4" s="21">
+        <v>0</v>
+      </c>
+      <c r="AI4" s="21">
+        <v>328.47</v>
+      </c>
+      <c r="AJ4" s="21">
+        <v>0</v>
+      </c>
+      <c r="AK4" s="21">
+        <v>0</v>
+      </c>
+      <c r="AL4" s="22">
+        <v>1</v>
+      </c>
+      <c r="AM4" s="21">
+        <v>4</v>
+      </c>
+      <c r="AN4" s="21">
+        <v>82.1175</v>
+      </c>
+      <c r="AO4" s="21">
+        <v>0</v>
+      </c>
+      <c r="AP4" s="21">
+        <v>0</v>
+      </c>
+      <c r="AQ4" s="21" t="s">
+        <v>76</v>
+      </c>
+      <c r="AR4" s="21">
+        <v>82.1175</v>
+      </c>
+      <c r="AS4" s="27" t="s">
+        <v>101</v>
+      </c>
+      <c r="AT4" s="28" t="s">
+        <v>76</v>
+      </c>
+      <c r="AU4" s="29" t="s">
+        <v>113</v>
+      </c>
+      <c r="AV4" s="29" t="s">
+        <v>114</v>
+      </c>
+      <c r="AW4" s="28">
+        <v>4</v>
+      </c>
+      <c r="AX4" s="28">
+        <v>82.1175</v>
+      </c>
+      <c r="AY4" s="28">
+        <v>52</v>
+      </c>
+      <c r="AZ4" s="28">
+        <v>82.12</v>
+      </c>
+      <c r="BA4" s="32"/>
+      <c r="BB4" s="32" t="s">
+        <v>80</v>
+      </c>
+      <c r="BC4" s="33" t="s">
+        <v>81</v>
+      </c>
+      <c r="BD4" s="34" t="s">
+        <v>82</v>
+      </c>
+      <c r="BE4" s="34" t="s">
+        <v>83</v>
+      </c>
+      <c r="BF4" s="32"/>
+      <c r="BG4" s="32"/>
+      <c r="BH4" s="32"/>
+      <c r="BI4" s="28"/>
+      <c r="BJ4" s="28"/>
+      <c r="BK4" s="28"/>
+      <c r="BL4" s="35" t="s">
+        <v>104</v>
+      </c>
+      <c r="BM4" s="29" t="s">
+        <v>114</v>
+      </c>
+      <c r="BN4" s="29" t="s">
+        <v>115</v>
+      </c>
+      <c r="BO4" s="28">
+        <v>82.12</v>
+      </c>
+      <c r="BP4" s="36">
+        <v>56</v>
+      </c>
+      <c r="BQ4" s="37">
+        <v>123562</v>
+      </c>
+    </row>
+    <row r="5" ht="15.25" spans="1:69">
+      <c r="A5" s="9"/>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="E5" s="11"/>
+      <c r="F5" s="11"/>
+      <c r="G5" s="12"/>
+      <c r="H5" s="13">
+        <f>SUM(H4:H4)</f>
+        <v>400</v>
+      </c>
+      <c r="I5" s="7"/>
+      <c r="J5" s="7"/>
+      <c r="K5" s="7"/>
+      <c r="L5" s="7"/>
+      <c r="M5" s="7"/>
+      <c r="N5" s="7"/>
+      <c r="O5" s="7"/>
+      <c r="P5" s="7"/>
+      <c r="Q5" s="7"/>
+      <c r="R5" s="13">
+        <f t="shared" ref="R5:AK5" si="0">SUM(R4:R4)</f>
+        <v>71.53</v>
+      </c>
+      <c r="S5" s="13">
+        <f t="shared" si="0"/>
+        <v>328.47</v>
+      </c>
+      <c r="T5" s="18"/>
+      <c r="U5" s="18"/>
+      <c r="V5" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="W5" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="X5" s="13">
+        <f t="shared" si="0"/>
+        <v>59.12</v>
+      </c>
+      <c r="Y5" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="Z5" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AA5" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AB5" s="13">
+        <f t="shared" si="0"/>
+        <v>59.12</v>
+      </c>
+      <c r="AC5" s="13">
+        <f t="shared" si="0"/>
+        <v>328.47</v>
+      </c>
+      <c r="AD5" s="13">
+        <f t="shared" si="0"/>
+        <v>120</v>
+      </c>
+      <c r="AE5" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AF5" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AG5" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AH5" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AI5" s="13">
+        <f t="shared" si="0"/>
+        <v>328.47</v>
+      </c>
+      <c r="AJ5" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AK5" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AL5" s="23"/>
+      <c r="AM5" s="23"/>
+      <c r="AN5" s="23"/>
+      <c r="AO5" s="23"/>
+      <c r="AP5" s="23"/>
+      <c r="AQ5" s="23"/>
+      <c r="AR5" s="23"/>
+      <c r="AS5" s="9"/>
+      <c r="AT5" s="9"/>
+      <c r="AU5" s="30"/>
+      <c r="AV5" s="30"/>
+      <c r="AW5" s="9"/>
+      <c r="AX5" s="9"/>
+      <c r="AY5" s="9"/>
+      <c r="AZ5" s="9"/>
+      <c r="BA5" s="9"/>
+      <c r="BB5" s="9"/>
+      <c r="BC5" s="9"/>
+      <c r="BD5" s="9"/>
+      <c r="BE5" s="9"/>
+      <c r="BF5" s="9"/>
+      <c r="BG5" s="9"/>
+      <c r="BH5" s="9"/>
+      <c r="BI5" s="9"/>
+      <c r="BJ5" s="9"/>
+      <c r="BK5" s="9"/>
+      <c r="BL5" s="9"/>
+      <c r="BM5" s="9"/>
+      <c r="BN5" s="9"/>
+      <c r="BO5" s="9"/>
+      <c r="BP5" s="30"/>
+      <c r="BQ5" s="30"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:B2"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="AS4" r:id="rId1" display="INS WH-1" tooltip="https://webappqc.roadmaperp.com:8765/ords/r/rmqc27/scm-us9011/warehouse1?p367019101_rowid=AAATkUAAHAADnkPAAX&amp;p367019101_store_id=INS WH-1&amp;session=1523407412914"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:BQ5"/>
+  <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5" outlineLevelRow="4"/>
+  <sheetData>
+    <row r="1" spans="1:69">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="14"/>
+      <c r="K1" s="14"/>
+      <c r="L1" s="14"/>
+      <c r="M1" s="14"/>
+      <c r="N1" s="14"/>
+      <c r="O1" s="14"/>
+      <c r="P1" s="14"/>
+      <c r="Q1" s="14"/>
+      <c r="R1" s="1"/>
+      <c r="S1" s="1"/>
+      <c r="T1" s="1"/>
+      <c r="U1" s="1"/>
+      <c r="V1" s="9"/>
+      <c r="W1" s="9"/>
+      <c r="X1" s="9"/>
+      <c r="Y1" s="9"/>
+      <c r="Z1" s="9"/>
+      <c r="AA1" s="9"/>
+      <c r="AB1" s="9"/>
+      <c r="AC1" s="9"/>
+      <c r="AD1" s="9"/>
+      <c r="AE1" s="9"/>
+      <c r="AF1" s="9"/>
+      <c r="AG1" s="9"/>
+      <c r="AH1" s="9"/>
+      <c r="AI1" s="9"/>
+      <c r="AJ1" s="9"/>
+      <c r="AK1" s="9"/>
+      <c r="AL1" s="9"/>
+      <c r="AM1" s="9"/>
+      <c r="AN1" s="9"/>
+      <c r="AO1" s="9"/>
+      <c r="AP1" s="9"/>
+      <c r="AQ1" s="9"/>
+      <c r="AR1" s="9"/>
+      <c r="AS1" s="9"/>
+      <c r="AT1" s="9"/>
+      <c r="AU1" s="9"/>
+      <c r="AV1" s="9"/>
+      <c r="AW1" s="9"/>
+      <c r="AX1" s="9"/>
+      <c r="AY1" s="9"/>
+      <c r="AZ1" s="9"/>
+      <c r="BA1" s="9"/>
+      <c r="BB1" s="9"/>
+      <c r="BC1" s="9"/>
+      <c r="BD1" s="9"/>
+      <c r="BE1" s="9"/>
+      <c r="BF1" s="9"/>
+      <c r="BG1" s="9"/>
+      <c r="BH1" s="9"/>
+      <c r="BI1" s="9"/>
+      <c r="BJ1" s="9"/>
+      <c r="BK1" s="9"/>
+      <c r="BL1" s="9"/>
+      <c r="BM1" s="9"/>
+      <c r="BN1" s="9"/>
+      <c r="BO1" s="9"/>
+      <c r="BP1" s="30"/>
+      <c r="BQ1" s="30"/>
+    </row>
+    <row r="2" ht="15.25" spans="1:69">
+      <c r="A2" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="4">
+        <v>2</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="J2" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="K2" s="14"/>
+      <c r="L2" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="M2" s="14">
+        <v>1</v>
+      </c>
+      <c r="N2" s="14"/>
+      <c r="O2" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="P2" s="14">
+        <v>2</v>
+      </c>
+      <c r="Q2" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="R2" s="1"/>
+      <c r="S2" s="1"/>
+      <c r="T2" s="1"/>
+      <c r="U2" s="1"/>
+      <c r="V2" s="1">
+        <v>1</v>
+      </c>
+      <c r="W2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="X2" s="9"/>
+      <c r="Y2" s="9"/>
+      <c r="Z2" s="9"/>
+      <c r="AA2" s="9"/>
+      <c r="AB2" s="9"/>
+      <c r="AC2" s="9"/>
+      <c r="AD2" s="9"/>
+      <c r="AE2" s="9"/>
+      <c r="AF2" s="9"/>
+      <c r="AG2" s="9"/>
+      <c r="AH2" s="9"/>
+      <c r="AI2" s="9"/>
+      <c r="AJ2" s="9"/>
+      <c r="AK2" s="9"/>
+      <c r="AL2" s="9"/>
+      <c r="AM2" s="9"/>
+      <c r="AN2" s="9"/>
+      <c r="AO2" s="9"/>
+      <c r="AP2" s="9"/>
+      <c r="AQ2" s="9"/>
+      <c r="AR2" s="9"/>
+      <c r="AS2" s="9"/>
+      <c r="AT2" s="9"/>
+      <c r="AU2" s="9"/>
+      <c r="AV2" s="9"/>
+      <c r="AW2" s="9"/>
+      <c r="AX2" s="9"/>
+      <c r="AY2" s="9"/>
+      <c r="AZ2" s="9"/>
+      <c r="BA2" s="9"/>
+      <c r="BB2" s="9"/>
+      <c r="BC2" s="9"/>
+      <c r="BD2" s="9"/>
+      <c r="BE2" s="9"/>
+      <c r="BF2" s="9"/>
+      <c r="BG2" s="9"/>
+      <c r="BH2" s="9"/>
+      <c r="BI2" s="9"/>
+      <c r="BJ2" s="9"/>
+      <c r="BK2" s="9"/>
+      <c r="BL2" s="9"/>
+      <c r="BM2" s="9"/>
+      <c r="BN2" s="9"/>
+      <c r="BO2" s="9"/>
+      <c r="BP2" s="30"/>
+      <c r="BQ2" s="30"/>
+    </row>
+    <row r="3" ht="45" spans="1:69">
+      <c r="A3" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="I3" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="J3" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="K3" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="L3" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="M3" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="N3" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="O3" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="P3" s="16" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q3" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="R3" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="S3" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="T3" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="U3" s="17" t="s">
+        <v>97</v>
+      </c>
+      <c r="V3" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="W3" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="X3" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="Y3" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="Z3" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="AA3" s="19" t="s">
+        <v>35</v>
+      </c>
+      <c r="AB3" s="19" t="s">
+        <v>36</v>
+      </c>
+      <c r="AC3" s="20" t="s">
+        <v>37</v>
+      </c>
+      <c r="AD3" s="20" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE3" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="AF3" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="AG3" s="20" t="s">
+        <v>41</v>
+      </c>
+      <c r="AH3" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="AI3" s="20" t="s">
+        <v>43</v>
+      </c>
+      <c r="AJ3" s="20" t="s">
+        <v>44</v>
+      </c>
+      <c r="AK3" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="AL3" s="20" t="s">
+        <v>46</v>
+      </c>
+      <c r="AM3" s="20" t="s">
+        <v>47</v>
+      </c>
+      <c r="AN3" s="20" t="s">
+        <v>48</v>
+      </c>
+      <c r="AO3" s="20" t="s">
+        <v>49</v>
+      </c>
+      <c r="AP3" s="20" t="s">
+        <v>50</v>
+      </c>
+      <c r="AQ3" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="AR3" s="24" t="s">
+        <v>98</v>
+      </c>
+      <c r="AS3" s="25" t="s">
+        <v>53</v>
+      </c>
+      <c r="AT3" s="25" t="s">
+        <v>51</v>
+      </c>
+      <c r="AU3" s="26" t="s">
+        <v>54</v>
+      </c>
+      <c r="AV3" s="26" t="s">
+        <v>55</v>
+      </c>
+      <c r="AW3" s="26" t="s">
+        <v>56</v>
+      </c>
+      <c r="AX3" s="26" t="s">
+        <v>57</v>
+      </c>
+      <c r="AY3" s="26" t="s">
+        <v>58</v>
+      </c>
+      <c r="AZ3" s="26" t="s">
+        <v>59</v>
+      </c>
+      <c r="BA3" s="26" t="s">
+        <v>60</v>
+      </c>
+      <c r="BB3" s="26" t="s">
+        <v>61</v>
+      </c>
+      <c r="BC3" s="31" t="s">
+        <v>62</v>
+      </c>
+      <c r="BD3" s="31" t="s">
+        <v>63</v>
+      </c>
+      <c r="BE3" s="31" t="s">
+        <v>64</v>
+      </c>
+      <c r="BF3" s="26" t="s">
+        <v>65</v>
+      </c>
+      <c r="BG3" s="26" t="s">
+        <v>66</v>
+      </c>
+      <c r="BH3" s="26" t="s">
+        <v>67</v>
+      </c>
+      <c r="BI3" s="26" t="s">
+        <v>68</v>
+      </c>
+      <c r="BJ3" s="26" t="s">
+        <v>69</v>
+      </c>
+      <c r="BK3" s="26" t="s">
+        <v>70</v>
+      </c>
+      <c r="BL3" s="26" t="s">
+        <v>71</v>
+      </c>
+      <c r="BM3" s="26" t="s">
+        <v>72</v>
+      </c>
+      <c r="BN3" s="26" t="s">
+        <v>73</v>
+      </c>
+      <c r="BO3" s="26" t="s">
+        <v>59</v>
+      </c>
+      <c r="BP3" s="26" t="s">
+        <v>74</v>
+      </c>
+      <c r="BQ3" s="26" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" ht="15.25" spans="1:69">
+      <c r="A4" s="7">
+        <v>1</v>
+      </c>
+      <c r="B4" s="7" t="s">
         <v>137</v>
       </c>
       <c r="C4" s="7" t="s">
         <v>137</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="F4" s="8">
+        <v>4</v>
+      </c>
+      <c r="G4" s="8">
+        <v>100</v>
+      </c>
+      <c r="H4" s="8">
+        <v>400</v>
+      </c>
+      <c r="I4" s="8">
+        <v>4</v>
+      </c>
+      <c r="J4" s="8">
+        <v>9</v>
+      </c>
+      <c r="K4" s="8">
+        <v>6</v>
+      </c>
+      <c r="L4" s="8">
+        <v>400</v>
+      </c>
+      <c r="M4" s="8">
+        <v>16</v>
+      </c>
+      <c r="N4" s="8">
+        <v>384</v>
+      </c>
+      <c r="O4" s="8">
+        <v>34.56</v>
+      </c>
+      <c r="P4" s="8">
+        <v>349.44</v>
+      </c>
+      <c r="Q4" s="8">
+        <v>20.97</v>
+      </c>
+      <c r="R4" s="8">
+        <v>71.53</v>
+      </c>
+      <c r="S4" s="8">
+        <v>328.47</v>
+      </c>
+      <c r="T4" s="8">
+        <v>88363222</v>
+      </c>
+      <c r="U4" s="8">
+        <v>18</v>
+      </c>
+      <c r="V4" s="8">
+        <v>0</v>
+      </c>
+      <c r="W4" s="8">
+        <v>0</v>
+      </c>
+      <c r="X4" s="8">
+        <v>59.12</v>
+      </c>
+      <c r="Y4" s="8">
+        <v>0</v>
+      </c>
+      <c r="Z4" s="8">
+        <v>0</v>
+      </c>
+      <c r="AA4" s="8">
+        <v>0</v>
+      </c>
+      <c r="AB4" s="8">
+        <v>59.12</v>
+      </c>
+      <c r="AC4" s="8">
+        <v>328.47</v>
+      </c>
+      <c r="AD4" s="21">
+        <v>120</v>
+      </c>
+      <c r="AE4" s="21">
+        <v>0</v>
+      </c>
+      <c r="AF4" s="21"/>
+      <c r="AG4" s="21">
+        <v>0</v>
+      </c>
+      <c r="AH4" s="21">
+        <v>0</v>
+      </c>
+      <c r="AI4" s="21">
+        <v>328.47</v>
+      </c>
+      <c r="AJ4" s="21">
+        <v>0</v>
+      </c>
+      <c r="AK4" s="21">
+        <v>0</v>
+      </c>
+      <c r="AL4" s="22">
+        <v>1</v>
+      </c>
+      <c r="AM4" s="21">
+        <v>4</v>
+      </c>
+      <c r="AN4" s="21">
+        <v>82.1175</v>
+      </c>
+      <c r="AO4" s="21">
+        <v>0</v>
+      </c>
+      <c r="AP4" s="21">
+        <v>0</v>
+      </c>
+      <c r="AQ4" s="21" t="s">
+        <v>76</v>
+      </c>
+      <c r="AR4" s="21">
+        <v>82.1175</v>
+      </c>
+      <c r="AS4" s="27" t="s">
+        <v>101</v>
+      </c>
+      <c r="AT4" s="28" t="s">
+        <v>76</v>
+      </c>
+      <c r="AU4" s="29" t="s">
+        <v>113</v>
+      </c>
+      <c r="AV4" s="29" t="s">
+        <v>114</v>
+      </c>
+      <c r="AW4" s="28">
+        <v>4</v>
+      </c>
+      <c r="AX4" s="28">
+        <v>82.1175</v>
+      </c>
+      <c r="AY4" s="28">
+        <v>52</v>
+      </c>
+      <c r="AZ4" s="28">
+        <v>82.12</v>
+      </c>
+      <c r="BA4" s="32"/>
+      <c r="BB4" s="32" t="s">
+        <v>80</v>
+      </c>
+      <c r="BC4" s="33" t="s">
+        <v>81</v>
+      </c>
+      <c r="BD4" s="34" t="s">
+        <v>82</v>
+      </c>
+      <c r="BE4" s="34" t="s">
+        <v>83</v>
+      </c>
+      <c r="BF4" s="32"/>
+      <c r="BG4" s="32"/>
+      <c r="BH4" s="32"/>
+      <c r="BI4" s="28"/>
+      <c r="BJ4" s="28"/>
+      <c r="BK4" s="28"/>
+      <c r="BL4" s="35" t="s">
+        <v>104</v>
+      </c>
+      <c r="BM4" s="29" t="s">
+        <v>114</v>
+      </c>
+      <c r="BN4" s="29" t="s">
+        <v>115</v>
+      </c>
+      <c r="BO4" s="28">
+        <v>82.12</v>
+      </c>
+      <c r="BP4" s="36">
+        <v>56</v>
+      </c>
+      <c r="BQ4" s="37">
+        <v>123562</v>
+      </c>
+    </row>
+    <row r="5" ht="15.25" spans="1:69">
+      <c r="A5" s="9"/>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="E5" s="11"/>
+      <c r="F5" s="11"/>
+      <c r="G5" s="12"/>
+      <c r="H5" s="13">
+        <f>SUM(H4:H4)</f>
+        <v>400</v>
+      </c>
+      <c r="I5" s="7"/>
+      <c r="J5" s="7"/>
+      <c r="K5" s="7"/>
+      <c r="L5" s="7"/>
+      <c r="M5" s="7"/>
+      <c r="N5" s="7"/>
+      <c r="O5" s="7"/>
+      <c r="P5" s="7"/>
+      <c r="Q5" s="7"/>
+      <c r="R5" s="13">
+        <f t="shared" ref="R5:AK5" si="0">SUM(R4:R4)</f>
+        <v>71.53</v>
+      </c>
+      <c r="S5" s="13">
+        <f t="shared" si="0"/>
+        <v>328.47</v>
+      </c>
+      <c r="T5" s="18"/>
+      <c r="U5" s="18"/>
+      <c r="V5" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="W5" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="X5" s="13">
+        <f t="shared" si="0"/>
+        <v>59.12</v>
+      </c>
+      <c r="Y5" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="Z5" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AA5" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AB5" s="13">
+        <f t="shared" si="0"/>
+        <v>59.12</v>
+      </c>
+      <c r="AC5" s="13">
+        <f t="shared" si="0"/>
+        <v>328.47</v>
+      </c>
+      <c r="AD5" s="13">
+        <f t="shared" si="0"/>
+        <v>120</v>
+      </c>
+      <c r="AE5" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AF5" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AG5" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AH5" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AI5" s="13">
+        <f t="shared" si="0"/>
+        <v>328.47</v>
+      </c>
+      <c r="AJ5" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AK5" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AL5" s="23"/>
+      <c r="AM5" s="23"/>
+      <c r="AN5" s="23"/>
+      <c r="AO5" s="23"/>
+      <c r="AP5" s="23"/>
+      <c r="AQ5" s="23"/>
+      <c r="AR5" s="23"/>
+      <c r="AS5" s="9"/>
+      <c r="AT5" s="9"/>
+      <c r="AU5" s="30"/>
+      <c r="AV5" s="30"/>
+      <c r="AW5" s="9"/>
+      <c r="AX5" s="9"/>
+      <c r="AY5" s="9"/>
+      <c r="AZ5" s="9"/>
+      <c r="BA5" s="9"/>
+      <c r="BB5" s="9"/>
+      <c r="BC5" s="9"/>
+      <c r="BD5" s="9"/>
+      <c r="BE5" s="9"/>
+      <c r="BF5" s="9"/>
+      <c r="BG5" s="9"/>
+      <c r="BH5" s="9"/>
+      <c r="BI5" s="9"/>
+      <c r="BJ5" s="9"/>
+      <c r="BK5" s="9"/>
+      <c r="BL5" s="9"/>
+      <c r="BM5" s="9"/>
+      <c r="BN5" s="9"/>
+      <c r="BO5" s="9"/>
+      <c r="BP5" s="30"/>
+      <c r="BQ5" s="30"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:B2"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="AS4" r:id="rId1" display="INS WH-1" tooltip="https://webappqc.roadmaperp.com:8765/ords/r/rmqc27/scm-us9011/warehouse1?p367019101_rowid=AAATkUAAHAADnkPAAX&amp;p367019101_store_id=INS WH-1&amp;session=1523407412914"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:BQ5"/>
+  <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5" outlineLevelRow="4"/>
+  <sheetData>
+    <row r="1" spans="1:69">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="14"/>
+      <c r="K1" s="14"/>
+      <c r="L1" s="14"/>
+      <c r="M1" s="14"/>
+      <c r="N1" s="14"/>
+      <c r="O1" s="14"/>
+      <c r="P1" s="14"/>
+      <c r="Q1" s="14"/>
+      <c r="R1" s="1"/>
+      <c r="S1" s="1"/>
+      <c r="T1" s="1"/>
+      <c r="U1" s="1"/>
+      <c r="V1" s="9"/>
+      <c r="W1" s="9"/>
+      <c r="X1" s="9"/>
+      <c r="Y1" s="9"/>
+      <c r="Z1" s="9"/>
+      <c r="AA1" s="9"/>
+      <c r="AB1" s="9"/>
+      <c r="AC1" s="9"/>
+      <c r="AD1" s="9"/>
+      <c r="AE1" s="9"/>
+      <c r="AF1" s="9"/>
+      <c r="AG1" s="9"/>
+      <c r="AH1" s="9"/>
+      <c r="AI1" s="9"/>
+      <c r="AJ1" s="9"/>
+      <c r="AK1" s="9"/>
+      <c r="AL1" s="9"/>
+      <c r="AM1" s="9"/>
+      <c r="AN1" s="9"/>
+      <c r="AO1" s="9"/>
+      <c r="AP1" s="9"/>
+      <c r="AQ1" s="9"/>
+      <c r="AR1" s="9"/>
+      <c r="AS1" s="9"/>
+      <c r="AT1" s="9"/>
+      <c r="AU1" s="9"/>
+      <c r="AV1" s="9"/>
+      <c r="AW1" s="9"/>
+      <c r="AX1" s="9"/>
+      <c r="AY1" s="9"/>
+      <c r="AZ1" s="9"/>
+      <c r="BA1" s="9"/>
+      <c r="BB1" s="9"/>
+      <c r="BC1" s="9"/>
+      <c r="BD1" s="9"/>
+      <c r="BE1" s="9"/>
+      <c r="BF1" s="9"/>
+      <c r="BG1" s="9"/>
+      <c r="BH1" s="9"/>
+      <c r="BI1" s="9"/>
+      <c r="BJ1" s="9"/>
+      <c r="BK1" s="9"/>
+      <c r="BL1" s="9"/>
+      <c r="BM1" s="9"/>
+      <c r="BN1" s="9"/>
+      <c r="BO1" s="9"/>
+      <c r="BP1" s="30"/>
+      <c r="BQ1" s="30"/>
+    </row>
+    <row r="2" ht="15.25" spans="1:69">
+      <c r="A2" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="4">
+        <v>2</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="J2" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="K2" s="14"/>
+      <c r="L2" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="M2" s="14">
+        <v>1</v>
+      </c>
+      <c r="N2" s="14"/>
+      <c r="O2" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="P2" s="14">
+        <v>2</v>
+      </c>
+      <c r="Q2" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="R2" s="1"/>
+      <c r="S2" s="1"/>
+      <c r="T2" s="1"/>
+      <c r="U2" s="1"/>
+      <c r="V2" s="1">
+        <v>1</v>
+      </c>
+      <c r="W2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="X2" s="9"/>
+      <c r="Y2" s="9"/>
+      <c r="Z2" s="9"/>
+      <c r="AA2" s="9"/>
+      <c r="AB2" s="9"/>
+      <c r="AC2" s="9"/>
+      <c r="AD2" s="9"/>
+      <c r="AE2" s="9"/>
+      <c r="AF2" s="9"/>
+      <c r="AG2" s="9"/>
+      <c r="AH2" s="9"/>
+      <c r="AI2" s="9"/>
+      <c r="AJ2" s="9"/>
+      <c r="AK2" s="9"/>
+      <c r="AL2" s="9"/>
+      <c r="AM2" s="9"/>
+      <c r="AN2" s="9"/>
+      <c r="AO2" s="9"/>
+      <c r="AP2" s="9"/>
+      <c r="AQ2" s="9"/>
+      <c r="AR2" s="9"/>
+      <c r="AS2" s="9"/>
+      <c r="AT2" s="9"/>
+      <c r="AU2" s="9"/>
+      <c r="AV2" s="9"/>
+      <c r="AW2" s="9"/>
+      <c r="AX2" s="9"/>
+      <c r="AY2" s="9"/>
+      <c r="AZ2" s="9"/>
+      <c r="BA2" s="9"/>
+      <c r="BB2" s="9"/>
+      <c r="BC2" s="9"/>
+      <c r="BD2" s="9"/>
+      <c r="BE2" s="9"/>
+      <c r="BF2" s="9"/>
+      <c r="BG2" s="9"/>
+      <c r="BH2" s="9"/>
+      <c r="BI2" s="9"/>
+      <c r="BJ2" s="9"/>
+      <c r="BK2" s="9"/>
+      <c r="BL2" s="9"/>
+      <c r="BM2" s="9"/>
+      <c r="BN2" s="9"/>
+      <c r="BO2" s="9"/>
+      <c r="BP2" s="30"/>
+      <c r="BQ2" s="30"/>
+    </row>
+    <row r="3" ht="45" spans="1:69">
+      <c r="A3" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="I3" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="J3" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="K3" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="L3" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="M3" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="N3" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="O3" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="P3" s="16" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q3" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="R3" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="S3" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="T3" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="U3" s="17" t="s">
+        <v>97</v>
+      </c>
+      <c r="V3" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="W3" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="X3" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="Y3" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="Z3" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="AA3" s="19" t="s">
+        <v>35</v>
+      </c>
+      <c r="AB3" s="19" t="s">
+        <v>36</v>
+      </c>
+      <c r="AC3" s="20" t="s">
+        <v>37</v>
+      </c>
+      <c r="AD3" s="20" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE3" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="AF3" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="AG3" s="20" t="s">
+        <v>41</v>
+      </c>
+      <c r="AH3" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="AI3" s="20" t="s">
+        <v>43</v>
+      </c>
+      <c r="AJ3" s="20" t="s">
+        <v>44</v>
+      </c>
+      <c r="AK3" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="AL3" s="20" t="s">
+        <v>46</v>
+      </c>
+      <c r="AM3" s="20" t="s">
+        <v>47</v>
+      </c>
+      <c r="AN3" s="20" t="s">
+        <v>48</v>
+      </c>
+      <c r="AO3" s="20" t="s">
+        <v>49</v>
+      </c>
+      <c r="AP3" s="20" t="s">
+        <v>50</v>
+      </c>
+      <c r="AQ3" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="AR3" s="24" t="s">
+        <v>98</v>
+      </c>
+      <c r="AS3" s="25" t="s">
+        <v>53</v>
+      </c>
+      <c r="AT3" s="25" t="s">
+        <v>51</v>
+      </c>
+      <c r="AU3" s="26" t="s">
+        <v>54</v>
+      </c>
+      <c r="AV3" s="26" t="s">
+        <v>55</v>
+      </c>
+      <c r="AW3" s="26" t="s">
+        <v>56</v>
+      </c>
+      <c r="AX3" s="26" t="s">
+        <v>57</v>
+      </c>
+      <c r="AY3" s="26" t="s">
+        <v>58</v>
+      </c>
+      <c r="AZ3" s="26" t="s">
+        <v>59</v>
+      </c>
+      <c r="BA3" s="26" t="s">
+        <v>60</v>
+      </c>
+      <c r="BB3" s="26" t="s">
+        <v>61</v>
+      </c>
+      <c r="BC3" s="31" t="s">
+        <v>62</v>
+      </c>
+      <c r="BD3" s="31" t="s">
+        <v>63</v>
+      </c>
+      <c r="BE3" s="31" t="s">
+        <v>64</v>
+      </c>
+      <c r="BF3" s="26" t="s">
+        <v>65</v>
+      </c>
+      <c r="BG3" s="26" t="s">
+        <v>66</v>
+      </c>
+      <c r="BH3" s="26" t="s">
+        <v>67</v>
+      </c>
+      <c r="BI3" s="26" t="s">
+        <v>68</v>
+      </c>
+      <c r="BJ3" s="26" t="s">
+        <v>69</v>
+      </c>
+      <c r="BK3" s="26" t="s">
+        <v>70</v>
+      </c>
+      <c r="BL3" s="26" t="s">
+        <v>71</v>
+      </c>
+      <c r="BM3" s="26" t="s">
+        <v>72</v>
+      </c>
+      <c r="BN3" s="26" t="s">
+        <v>73</v>
+      </c>
+      <c r="BO3" s="26" t="s">
+        <v>59</v>
+      </c>
+      <c r="BP3" s="26" t="s">
+        <v>74</v>
+      </c>
+      <c r="BQ3" s="26" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" ht="15.25" spans="1:69">
+      <c r="A4" s="7">
+        <v>1</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="F4" s="8">
+        <v>4</v>
+      </c>
+      <c r="G4" s="8">
+        <v>100</v>
+      </c>
+      <c r="H4" s="8">
+        <v>400</v>
+      </c>
+      <c r="I4" s="8">
+        <v>4</v>
+      </c>
+      <c r="J4" s="8">
+        <v>9</v>
+      </c>
+      <c r="K4" s="8">
+        <v>6</v>
+      </c>
+      <c r="L4" s="8">
+        <v>400</v>
+      </c>
+      <c r="M4" s="8">
+        <v>16</v>
+      </c>
+      <c r="N4" s="8">
+        <v>384</v>
+      </c>
+      <c r="O4" s="8">
+        <v>34.56</v>
+      </c>
+      <c r="P4" s="8">
+        <v>349.44</v>
+      </c>
+      <c r="Q4" s="8">
+        <v>20.97</v>
+      </c>
+      <c r="R4" s="8">
+        <v>71.53</v>
+      </c>
+      <c r="S4" s="8">
+        <v>328.47</v>
+      </c>
+      <c r="T4" s="8">
+        <v>88363222</v>
+      </c>
+      <c r="U4" s="8">
+        <v>18</v>
+      </c>
+      <c r="V4" s="8">
+        <v>0</v>
+      </c>
+      <c r="W4" s="8">
+        <v>0</v>
+      </c>
+      <c r="X4" s="8">
+        <v>59.12</v>
+      </c>
+      <c r="Y4" s="8">
+        <v>0</v>
+      </c>
+      <c r="Z4" s="8">
+        <v>0</v>
+      </c>
+      <c r="AA4" s="8">
+        <v>0</v>
+      </c>
+      <c r="AB4" s="8">
+        <v>59.12</v>
+      </c>
+      <c r="AC4" s="8">
+        <v>328.47</v>
+      </c>
+      <c r="AD4" s="21">
+        <v>120</v>
+      </c>
+      <c r="AE4" s="21">
+        <v>0</v>
+      </c>
+      <c r="AF4" s="21"/>
+      <c r="AG4" s="21">
+        <v>0</v>
+      </c>
+      <c r="AH4" s="21">
+        <v>0</v>
+      </c>
+      <c r="AI4" s="21">
+        <v>328.47</v>
+      </c>
+      <c r="AJ4" s="21">
+        <v>0</v>
+      </c>
+      <c r="AK4" s="21">
+        <v>0</v>
+      </c>
+      <c r="AL4" s="22">
+        <v>1</v>
+      </c>
+      <c r="AM4" s="21">
+        <v>4</v>
+      </c>
+      <c r="AN4" s="21">
+        <v>82.1175</v>
+      </c>
+      <c r="AO4" s="21">
+        <v>0</v>
+      </c>
+      <c r="AP4" s="21">
+        <v>0</v>
+      </c>
+      <c r="AQ4" s="21" t="s">
+        <v>76</v>
+      </c>
+      <c r="AR4" s="21">
+        <v>82.1175</v>
+      </c>
+      <c r="AS4" s="27" t="s">
+        <v>101</v>
+      </c>
+      <c r="AT4" s="28" t="s">
+        <v>76</v>
+      </c>
+      <c r="AU4" s="29" t="s">
+        <v>113</v>
+      </c>
+      <c r="AV4" s="29" t="s">
+        <v>114</v>
+      </c>
+      <c r="AW4" s="28">
+        <v>4</v>
+      </c>
+      <c r="AX4" s="28">
+        <v>82.1175</v>
+      </c>
+      <c r="AY4" s="28">
+        <v>52</v>
+      </c>
+      <c r="AZ4" s="28">
+        <v>82.12</v>
+      </c>
+      <c r="BA4" s="32"/>
+      <c r="BB4" s="32" t="s">
+        <v>80</v>
+      </c>
+      <c r="BC4" s="33" t="s">
+        <v>81</v>
+      </c>
+      <c r="BD4" s="34" t="s">
+        <v>82</v>
+      </c>
+      <c r="BE4" s="34" t="s">
+        <v>83</v>
+      </c>
+      <c r="BF4" s="32"/>
+      <c r="BG4" s="32"/>
+      <c r="BH4" s="32"/>
+      <c r="BI4" s="28"/>
+      <c r="BJ4" s="28"/>
+      <c r="BK4" s="28"/>
+      <c r="BL4" s="35" t="s">
+        <v>104</v>
+      </c>
+      <c r="BM4" s="29" t="s">
+        <v>114</v>
+      </c>
+      <c r="BN4" s="29" t="s">
+        <v>115</v>
+      </c>
+      <c r="BO4" s="28">
+        <v>82.12</v>
+      </c>
+      <c r="BP4" s="36">
+        <v>56</v>
+      </c>
+      <c r="BQ4" s="37">
+        <v>123562</v>
+      </c>
+    </row>
+    <row r="5" ht="15.25" spans="1:69">
+      <c r="A5" s="9"/>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="E5" s="11"/>
+      <c r="F5" s="11"/>
+      <c r="G5" s="12"/>
+      <c r="H5" s="13">
+        <f>SUM(H4:H4)</f>
+        <v>400</v>
+      </c>
+      <c r="I5" s="7"/>
+      <c r="J5" s="7"/>
+      <c r="K5" s="7"/>
+      <c r="L5" s="7"/>
+      <c r="M5" s="7"/>
+      <c r="N5" s="7"/>
+      <c r="O5" s="7"/>
+      <c r="P5" s="7"/>
+      <c r="Q5" s="7"/>
+      <c r="R5" s="13">
+        <f t="shared" ref="R5:AK5" si="0">SUM(R4:R4)</f>
+        <v>71.53</v>
+      </c>
+      <c r="S5" s="13">
+        <f t="shared" si="0"/>
+        <v>328.47</v>
+      </c>
+      <c r="T5" s="18"/>
+      <c r="U5" s="18"/>
+      <c r="V5" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="W5" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="X5" s="13">
+        <f t="shared" si="0"/>
+        <v>59.12</v>
+      </c>
+      <c r="Y5" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="Z5" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AA5" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AB5" s="13">
+        <f t="shared" si="0"/>
+        <v>59.12</v>
+      </c>
+      <c r="AC5" s="13">
+        <f t="shared" si="0"/>
+        <v>328.47</v>
+      </c>
+      <c r="AD5" s="13">
+        <f t="shared" si="0"/>
+        <v>120</v>
+      </c>
+      <c r="AE5" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AF5" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AG5" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AH5" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AI5" s="13">
+        <f t="shared" si="0"/>
+        <v>328.47</v>
+      </c>
+      <c r="AJ5" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AK5" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AL5" s="23"/>
+      <c r="AM5" s="23"/>
+      <c r="AN5" s="23"/>
+      <c r="AO5" s="23"/>
+      <c r="AP5" s="23"/>
+      <c r="AQ5" s="23"/>
+      <c r="AR5" s="23"/>
+      <c r="AS5" s="9"/>
+      <c r="AT5" s="9"/>
+      <c r="AU5" s="30"/>
+      <c r="AV5" s="30"/>
+      <c r="AW5" s="9"/>
+      <c r="AX5" s="9"/>
+      <c r="AY5" s="9"/>
+      <c r="AZ5" s="9"/>
+      <c r="BA5" s="9"/>
+      <c r="BB5" s="9"/>
+      <c r="BC5" s="9"/>
+      <c r="BD5" s="9"/>
+      <c r="BE5" s="9"/>
+      <c r="BF5" s="9"/>
+      <c r="BG5" s="9"/>
+      <c r="BH5" s="9"/>
+      <c r="BI5" s="9"/>
+      <c r="BJ5" s="9"/>
+      <c r="BK5" s="9"/>
+      <c r="BL5" s="9"/>
+      <c r="BM5" s="9"/>
+      <c r="BN5" s="9"/>
+      <c r="BO5" s="9"/>
+      <c r="BP5" s="30"/>
+      <c r="BQ5" s="30"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:B2"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="AS4" r:id="rId1" display="INS WH-1" tooltip="https://webappqc.roadmaperp.com:8765/ords/r/rmqc27/scm-us9011/warehouse1?p367019101_rowid=AAATkUAAHAADnkPAAX&amp;p367019101_store_id=INS WH-1&amp;session=1523407412914"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:BQ5"/>
+  <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5" outlineLevelRow="4"/>
+  <cols>
+    <col min="2" max="2" width="28.2727272727273" customWidth="1"/>
+    <col min="3" max="3" width="24.9090909090909" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:69">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="14"/>
+      <c r="K1" s="14"/>
+      <c r="L1" s="14"/>
+      <c r="M1" s="14"/>
+      <c r="N1" s="14"/>
+      <c r="O1" s="14"/>
+      <c r="P1" s="14"/>
+      <c r="Q1" s="14"/>
+      <c r="R1" s="1"/>
+      <c r="S1" s="1"/>
+      <c r="T1" s="1"/>
+      <c r="U1" s="1"/>
+      <c r="V1" s="9"/>
+      <c r="W1" s="9"/>
+      <c r="X1" s="9"/>
+      <c r="Y1" s="9"/>
+      <c r="Z1" s="9"/>
+      <c r="AA1" s="9"/>
+      <c r="AB1" s="9"/>
+      <c r="AC1" s="9"/>
+      <c r="AD1" s="9"/>
+      <c r="AE1" s="9"/>
+      <c r="AF1" s="9"/>
+      <c r="AG1" s="9"/>
+      <c r="AH1" s="9"/>
+      <c r="AI1" s="9"/>
+      <c r="AJ1" s="9"/>
+      <c r="AK1" s="9"/>
+      <c r="AL1" s="9"/>
+      <c r="AM1" s="9"/>
+      <c r="AN1" s="9"/>
+      <c r="AO1" s="9"/>
+      <c r="AP1" s="9"/>
+      <c r="AQ1" s="9"/>
+      <c r="AR1" s="9"/>
+      <c r="AS1" s="9"/>
+      <c r="AT1" s="9"/>
+      <c r="AU1" s="9"/>
+      <c r="AV1" s="9"/>
+      <c r="AW1" s="9"/>
+      <c r="AX1" s="9"/>
+      <c r="AY1" s="9"/>
+      <c r="AZ1" s="9"/>
+      <c r="BA1" s="9"/>
+      <c r="BB1" s="9"/>
+      <c r="BC1" s="9"/>
+      <c r="BD1" s="9"/>
+      <c r="BE1" s="9"/>
+      <c r="BF1" s="9"/>
+      <c r="BG1" s="9"/>
+      <c r="BH1" s="9"/>
+      <c r="BI1" s="9"/>
+      <c r="BJ1" s="9"/>
+      <c r="BK1" s="9"/>
+      <c r="BL1" s="9"/>
+      <c r="BM1" s="9"/>
+      <c r="BN1" s="9"/>
+      <c r="BO1" s="9"/>
+      <c r="BP1" s="30"/>
+      <c r="BQ1" s="30"/>
+    </row>
+    <row r="2" ht="15.25" spans="1:69">
+      <c r="A2" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="4">
+        <v>2</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="J2" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="K2" s="14"/>
+      <c r="L2" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="M2" s="14">
+        <v>1</v>
+      </c>
+      <c r="N2" s="14"/>
+      <c r="O2" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="P2" s="14">
+        <v>2</v>
+      </c>
+      <c r="Q2" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="R2" s="1"/>
+      <c r="S2" s="1"/>
+      <c r="T2" s="1"/>
+      <c r="U2" s="1"/>
+      <c r="V2" s="1">
+        <v>1</v>
+      </c>
+      <c r="W2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="X2" s="9"/>
+      <c r="Y2" s="9"/>
+      <c r="Z2" s="9"/>
+      <c r="AA2" s="9"/>
+      <c r="AB2" s="9"/>
+      <c r="AC2" s="9"/>
+      <c r="AD2" s="9"/>
+      <c r="AE2" s="9"/>
+      <c r="AF2" s="9"/>
+      <c r="AG2" s="9"/>
+      <c r="AH2" s="9"/>
+      <c r="AI2" s="9"/>
+      <c r="AJ2" s="9"/>
+      <c r="AK2" s="9"/>
+      <c r="AL2" s="9"/>
+      <c r="AM2" s="9"/>
+      <c r="AN2" s="9"/>
+      <c r="AO2" s="9"/>
+      <c r="AP2" s="9"/>
+      <c r="AQ2" s="9"/>
+      <c r="AR2" s="9"/>
+      <c r="AS2" s="9"/>
+      <c r="AT2" s="9"/>
+      <c r="AU2" s="9"/>
+      <c r="AV2" s="9"/>
+      <c r="AW2" s="9"/>
+      <c r="AX2" s="9"/>
+      <c r="AY2" s="9"/>
+      <c r="AZ2" s="9"/>
+      <c r="BA2" s="9"/>
+      <c r="BB2" s="9"/>
+      <c r="BC2" s="9"/>
+      <c r="BD2" s="9"/>
+      <c r="BE2" s="9"/>
+      <c r="BF2" s="9"/>
+      <c r="BG2" s="9"/>
+      <c r="BH2" s="9"/>
+      <c r="BI2" s="9"/>
+      <c r="BJ2" s="9"/>
+      <c r="BK2" s="9"/>
+      <c r="BL2" s="9"/>
+      <c r="BM2" s="9"/>
+      <c r="BN2" s="9"/>
+      <c r="BO2" s="9"/>
+      <c r="BP2" s="30"/>
+      <c r="BQ2" s="30"/>
+    </row>
+    <row r="3" ht="45" spans="1:69">
+      <c r="A3" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="I3" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="J3" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="K3" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="L3" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="M3" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="N3" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="O3" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="P3" s="16" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q3" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="R3" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="S3" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="T3" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="U3" s="17" t="s">
+        <v>97</v>
+      </c>
+      <c r="V3" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="W3" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="X3" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="Y3" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="Z3" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="AA3" s="19" t="s">
+        <v>35</v>
+      </c>
+      <c r="AB3" s="19" t="s">
+        <v>36</v>
+      </c>
+      <c r="AC3" s="20" t="s">
+        <v>37</v>
+      </c>
+      <c r="AD3" s="20" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE3" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="AF3" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="AG3" s="20" t="s">
+        <v>41</v>
+      </c>
+      <c r="AH3" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="AI3" s="20" t="s">
+        <v>43</v>
+      </c>
+      <c r="AJ3" s="20" t="s">
+        <v>44</v>
+      </c>
+      <c r="AK3" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="AL3" s="20" t="s">
+        <v>46</v>
+      </c>
+      <c r="AM3" s="20" t="s">
+        <v>47</v>
+      </c>
+      <c r="AN3" s="20" t="s">
+        <v>48</v>
+      </c>
+      <c r="AO3" s="20" t="s">
+        <v>49</v>
+      </c>
+      <c r="AP3" s="20" t="s">
+        <v>50</v>
+      </c>
+      <c r="AQ3" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="AR3" s="24" t="s">
+        <v>98</v>
+      </c>
+      <c r="AS3" s="25" t="s">
+        <v>53</v>
+      </c>
+      <c r="AT3" s="25" t="s">
+        <v>51</v>
+      </c>
+      <c r="AU3" s="26" t="s">
+        <v>54</v>
+      </c>
+      <c r="AV3" s="26" t="s">
+        <v>55</v>
+      </c>
+      <c r="AW3" s="26" t="s">
+        <v>56</v>
+      </c>
+      <c r="AX3" s="26" t="s">
+        <v>57</v>
+      </c>
+      <c r="AY3" s="26" t="s">
+        <v>58</v>
+      </c>
+      <c r="AZ3" s="26" t="s">
+        <v>59</v>
+      </c>
+      <c r="BA3" s="26" t="s">
+        <v>60</v>
+      </c>
+      <c r="BB3" s="26" t="s">
+        <v>61</v>
+      </c>
+      <c r="BC3" s="31" t="s">
+        <v>62</v>
+      </c>
+      <c r="BD3" s="31" t="s">
+        <v>63</v>
+      </c>
+      <c r="BE3" s="31" t="s">
+        <v>64</v>
+      </c>
+      <c r="BF3" s="26" t="s">
+        <v>65</v>
+      </c>
+      <c r="BG3" s="26" t="s">
+        <v>66</v>
+      </c>
+      <c r="BH3" s="26" t="s">
+        <v>67</v>
+      </c>
+      <c r="BI3" s="26" t="s">
+        <v>68</v>
+      </c>
+      <c r="BJ3" s="26" t="s">
+        <v>69</v>
+      </c>
+      <c r="BK3" s="26" t="s">
+        <v>70</v>
+      </c>
+      <c r="BL3" s="26" t="s">
+        <v>71</v>
+      </c>
+      <c r="BM3" s="26" t="s">
+        <v>72</v>
+      </c>
+      <c r="BN3" s="26" t="s">
+        <v>73</v>
+      </c>
+      <c r="BO3" s="26" t="s">
+        <v>59</v>
+      </c>
+      <c r="BP3" s="26" t="s">
+        <v>74</v>
+      </c>
+      <c r="BQ3" s="26" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" ht="15.25" spans="1:69">
+      <c r="A4" s="7">
+        <v>1</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>126</v>
       </c>
       <c r="D4" s="7" t="s">
         <v>76</v>
@@ -24537,6 +26670,724 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:BQ5"/>
+  <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5" outlineLevelRow="4"/>
+  <sheetData>
+    <row r="1" spans="1:69">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="14"/>
+      <c r="K1" s="14"/>
+      <c r="L1" s="14"/>
+      <c r="M1" s="14"/>
+      <c r="N1" s="14"/>
+      <c r="O1" s="14"/>
+      <c r="P1" s="14"/>
+      <c r="Q1" s="14"/>
+      <c r="R1" s="1"/>
+      <c r="S1" s="1"/>
+      <c r="T1" s="1"/>
+      <c r="U1" s="1"/>
+      <c r="V1" s="9"/>
+      <c r="W1" s="9"/>
+      <c r="X1" s="9"/>
+      <c r="Y1" s="9"/>
+      <c r="Z1" s="9"/>
+      <c r="AA1" s="9"/>
+      <c r="AB1" s="9"/>
+      <c r="AC1" s="9"/>
+      <c r="AD1" s="9"/>
+      <c r="AE1" s="9"/>
+      <c r="AF1" s="9"/>
+      <c r="AG1" s="9"/>
+      <c r="AH1" s="9"/>
+      <c r="AI1" s="9"/>
+      <c r="AJ1" s="9"/>
+      <c r="AK1" s="9"/>
+      <c r="AL1" s="9"/>
+      <c r="AM1" s="9"/>
+      <c r="AN1" s="9"/>
+      <c r="AO1" s="9"/>
+      <c r="AP1" s="9"/>
+      <c r="AQ1" s="9"/>
+      <c r="AR1" s="9"/>
+      <c r="AS1" s="9"/>
+      <c r="AT1" s="9"/>
+      <c r="AU1" s="9"/>
+      <c r="AV1" s="9"/>
+      <c r="AW1" s="9"/>
+      <c r="AX1" s="9"/>
+      <c r="AY1" s="9"/>
+      <c r="AZ1" s="9"/>
+      <c r="BA1" s="9"/>
+      <c r="BB1" s="9"/>
+      <c r="BC1" s="9"/>
+      <c r="BD1" s="9"/>
+      <c r="BE1" s="9"/>
+      <c r="BF1" s="9"/>
+      <c r="BG1" s="9"/>
+      <c r="BH1" s="9"/>
+      <c r="BI1" s="9"/>
+      <c r="BJ1" s="9"/>
+      <c r="BK1" s="9"/>
+      <c r="BL1" s="9"/>
+      <c r="BM1" s="9"/>
+      <c r="BN1" s="9"/>
+      <c r="BO1" s="9"/>
+      <c r="BP1" s="30"/>
+      <c r="BQ1" s="30"/>
+    </row>
+    <row r="2" ht="15.25" spans="1:69">
+      <c r="A2" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="4">
+        <v>2</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="J2" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="K2" s="14"/>
+      <c r="L2" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="M2" s="14">
+        <v>1</v>
+      </c>
+      <c r="N2" s="14"/>
+      <c r="O2" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="P2" s="14">
+        <v>2</v>
+      </c>
+      <c r="Q2" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="R2" s="1"/>
+      <c r="S2" s="1"/>
+      <c r="T2" s="1"/>
+      <c r="U2" s="1"/>
+      <c r="V2" s="1">
+        <v>1</v>
+      </c>
+      <c r="W2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="X2" s="9"/>
+      <c r="Y2" s="9"/>
+      <c r="Z2" s="9"/>
+      <c r="AA2" s="9"/>
+      <c r="AB2" s="9"/>
+      <c r="AC2" s="9"/>
+      <c r="AD2" s="9"/>
+      <c r="AE2" s="9"/>
+      <c r="AF2" s="9"/>
+      <c r="AG2" s="9"/>
+      <c r="AH2" s="9"/>
+      <c r="AI2" s="9"/>
+      <c r="AJ2" s="9"/>
+      <c r="AK2" s="9"/>
+      <c r="AL2" s="9"/>
+      <c r="AM2" s="9"/>
+      <c r="AN2" s="9"/>
+      <c r="AO2" s="9"/>
+      <c r="AP2" s="9"/>
+      <c r="AQ2" s="9"/>
+      <c r="AR2" s="9"/>
+      <c r="AS2" s="9"/>
+      <c r="AT2" s="9"/>
+      <c r="AU2" s="9"/>
+      <c r="AV2" s="9"/>
+      <c r="AW2" s="9"/>
+      <c r="AX2" s="9"/>
+      <c r="AY2" s="9"/>
+      <c r="AZ2" s="9"/>
+      <c r="BA2" s="9"/>
+      <c r="BB2" s="9"/>
+      <c r="BC2" s="9"/>
+      <c r="BD2" s="9"/>
+      <c r="BE2" s="9"/>
+      <c r="BF2" s="9"/>
+      <c r="BG2" s="9"/>
+      <c r="BH2" s="9"/>
+      <c r="BI2" s="9"/>
+      <c r="BJ2" s="9"/>
+      <c r="BK2" s="9"/>
+      <c r="BL2" s="9"/>
+      <c r="BM2" s="9"/>
+      <c r="BN2" s="9"/>
+      <c r="BO2" s="9"/>
+      <c r="BP2" s="30"/>
+      <c r="BQ2" s="30"/>
+    </row>
+    <row r="3" ht="45" spans="1:69">
+      <c r="A3" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="I3" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="J3" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="K3" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="L3" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="M3" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="N3" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="O3" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="P3" s="16" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q3" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="R3" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="S3" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="T3" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="U3" s="17" t="s">
+        <v>97</v>
+      </c>
+      <c r="V3" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="W3" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="X3" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="Y3" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="Z3" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="AA3" s="19" t="s">
+        <v>35</v>
+      </c>
+      <c r="AB3" s="19" t="s">
+        <v>36</v>
+      </c>
+      <c r="AC3" s="20" t="s">
+        <v>37</v>
+      </c>
+      <c r="AD3" s="20" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE3" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="AF3" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="AG3" s="20" t="s">
+        <v>41</v>
+      </c>
+      <c r="AH3" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="AI3" s="20" t="s">
+        <v>43</v>
+      </c>
+      <c r="AJ3" s="20" t="s">
+        <v>44</v>
+      </c>
+      <c r="AK3" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="AL3" s="20" t="s">
+        <v>46</v>
+      </c>
+      <c r="AM3" s="20" t="s">
+        <v>47</v>
+      </c>
+      <c r="AN3" s="20" t="s">
+        <v>48</v>
+      </c>
+      <c r="AO3" s="20" t="s">
+        <v>49</v>
+      </c>
+      <c r="AP3" s="20" t="s">
+        <v>50</v>
+      </c>
+      <c r="AQ3" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="AR3" s="24" t="s">
+        <v>98</v>
+      </c>
+      <c r="AS3" s="25" t="s">
+        <v>53</v>
+      </c>
+      <c r="AT3" s="25" t="s">
+        <v>51</v>
+      </c>
+      <c r="AU3" s="26" t="s">
+        <v>54</v>
+      </c>
+      <c r="AV3" s="26" t="s">
+        <v>55</v>
+      </c>
+      <c r="AW3" s="26" t="s">
+        <v>56</v>
+      </c>
+      <c r="AX3" s="26" t="s">
+        <v>57</v>
+      </c>
+      <c r="AY3" s="26" t="s">
+        <v>58</v>
+      </c>
+      <c r="AZ3" s="26" t="s">
+        <v>59</v>
+      </c>
+      <c r="BA3" s="26" t="s">
+        <v>60</v>
+      </c>
+      <c r="BB3" s="26" t="s">
+        <v>61</v>
+      </c>
+      <c r="BC3" s="31" t="s">
+        <v>62</v>
+      </c>
+      <c r="BD3" s="31" t="s">
+        <v>63</v>
+      </c>
+      <c r="BE3" s="31" t="s">
+        <v>64</v>
+      </c>
+      <c r="BF3" s="26" t="s">
+        <v>65</v>
+      </c>
+      <c r="BG3" s="26" t="s">
+        <v>66</v>
+      </c>
+      <c r="BH3" s="26" t="s">
+        <v>67</v>
+      </c>
+      <c r="BI3" s="26" t="s">
+        <v>68</v>
+      </c>
+      <c r="BJ3" s="26" t="s">
+        <v>69</v>
+      </c>
+      <c r="BK3" s="26" t="s">
+        <v>70</v>
+      </c>
+      <c r="BL3" s="26" t="s">
+        <v>71</v>
+      </c>
+      <c r="BM3" s="26" t="s">
+        <v>72</v>
+      </c>
+      <c r="BN3" s="26" t="s">
+        <v>73</v>
+      </c>
+      <c r="BO3" s="26" t="s">
+        <v>59</v>
+      </c>
+      <c r="BP3" s="26" t="s">
+        <v>74</v>
+      </c>
+      <c r="BQ3" s="26" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" ht="15.25" spans="1:69">
+      <c r="A4" s="7">
+        <v>1</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="F4" s="8">
+        <v>4</v>
+      </c>
+      <c r="G4" s="8">
+        <v>100</v>
+      </c>
+      <c r="H4" s="8">
+        <v>400</v>
+      </c>
+      <c r="I4" s="8">
+        <v>4</v>
+      </c>
+      <c r="J4" s="8">
+        <v>9</v>
+      </c>
+      <c r="K4" s="8">
+        <v>6</v>
+      </c>
+      <c r="L4" s="8">
+        <v>400</v>
+      </c>
+      <c r="M4" s="8">
+        <v>16</v>
+      </c>
+      <c r="N4" s="8">
+        <v>384</v>
+      </c>
+      <c r="O4" s="8">
+        <v>34.56</v>
+      </c>
+      <c r="P4" s="8">
+        <v>349.44</v>
+      </c>
+      <c r="Q4" s="8">
+        <v>20.97</v>
+      </c>
+      <c r="R4" s="8">
+        <v>71.53</v>
+      </c>
+      <c r="S4" s="8">
+        <v>328.47</v>
+      </c>
+      <c r="T4" s="8">
+        <v>88363222</v>
+      </c>
+      <c r="U4" s="8">
+        <v>18</v>
+      </c>
+      <c r="V4" s="8">
+        <v>0</v>
+      </c>
+      <c r="W4" s="8">
+        <v>0</v>
+      </c>
+      <c r="X4" s="8">
+        <v>59.12</v>
+      </c>
+      <c r="Y4" s="8">
+        <v>0</v>
+      </c>
+      <c r="Z4" s="8">
+        <v>0</v>
+      </c>
+      <c r="AA4" s="8">
+        <v>0</v>
+      </c>
+      <c r="AB4" s="8">
+        <v>59.12</v>
+      </c>
+      <c r="AC4" s="8">
+        <v>328.47</v>
+      </c>
+      <c r="AD4" s="21">
+        <v>120</v>
+      </c>
+      <c r="AE4" s="21">
+        <v>0</v>
+      </c>
+      <c r="AF4" s="21"/>
+      <c r="AG4" s="21">
+        <v>0</v>
+      </c>
+      <c r="AH4" s="21">
+        <v>0</v>
+      </c>
+      <c r="AI4" s="21">
+        <v>328.47</v>
+      </c>
+      <c r="AJ4" s="21">
+        <v>0</v>
+      </c>
+      <c r="AK4" s="21">
+        <v>0</v>
+      </c>
+      <c r="AL4" s="22">
+        <v>1</v>
+      </c>
+      <c r="AM4" s="21">
+        <v>4</v>
+      </c>
+      <c r="AN4" s="21">
+        <v>82.1175</v>
+      </c>
+      <c r="AO4" s="21">
+        <v>0</v>
+      </c>
+      <c r="AP4" s="21">
+        <v>0</v>
+      </c>
+      <c r="AQ4" s="21" t="s">
+        <v>76</v>
+      </c>
+      <c r="AR4" s="21">
+        <v>82.1175</v>
+      </c>
+      <c r="AS4" s="27" t="s">
+        <v>101</v>
+      </c>
+      <c r="AT4" s="28" t="s">
+        <v>76</v>
+      </c>
+      <c r="AU4" s="29" t="s">
+        <v>113</v>
+      </c>
+      <c r="AV4" s="29" t="s">
+        <v>114</v>
+      </c>
+      <c r="AW4" s="28">
+        <v>4</v>
+      </c>
+      <c r="AX4" s="28">
+        <v>82.1175</v>
+      </c>
+      <c r="AY4" s="28">
+        <v>52</v>
+      </c>
+      <c r="AZ4" s="28">
+        <v>82.12</v>
+      </c>
+      <c r="BA4" s="32"/>
+      <c r="BB4" s="32" t="s">
+        <v>80</v>
+      </c>
+      <c r="BC4" s="33" t="s">
+        <v>81</v>
+      </c>
+      <c r="BD4" s="34" t="s">
+        <v>82</v>
+      </c>
+      <c r="BE4" s="34" t="s">
+        <v>83</v>
+      </c>
+      <c r="BF4" s="32"/>
+      <c r="BG4" s="32"/>
+      <c r="BH4" s="32"/>
+      <c r="BI4" s="28"/>
+      <c r="BJ4" s="28"/>
+      <c r="BK4" s="28"/>
+      <c r="BL4" s="35" t="s">
+        <v>104</v>
+      </c>
+      <c r="BM4" s="29" t="s">
+        <v>114</v>
+      </c>
+      <c r="BN4" s="29" t="s">
+        <v>115</v>
+      </c>
+      <c r="BO4" s="28">
+        <v>82.12</v>
+      </c>
+      <c r="BP4" s="36">
+        <v>56</v>
+      </c>
+      <c r="BQ4" s="37">
+        <v>123562</v>
+      </c>
+    </row>
+    <row r="5" ht="15.25" spans="1:69">
+      <c r="A5" s="9"/>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="E5" s="11"/>
+      <c r="F5" s="11"/>
+      <c r="G5" s="12"/>
+      <c r="H5" s="13">
+        <f>SUM(H4:H4)</f>
+        <v>400</v>
+      </c>
+      <c r="I5" s="7"/>
+      <c r="J5" s="7"/>
+      <c r="K5" s="7"/>
+      <c r="L5" s="7"/>
+      <c r="M5" s="7"/>
+      <c r="N5" s="7"/>
+      <c r="O5" s="7"/>
+      <c r="P5" s="7"/>
+      <c r="Q5" s="7"/>
+      <c r="R5" s="13">
+        <f t="shared" ref="R5:AK5" si="0">SUM(R4:R4)</f>
+        <v>71.53</v>
+      </c>
+      <c r="S5" s="13">
+        <f t="shared" si="0"/>
+        <v>328.47</v>
+      </c>
+      <c r="T5" s="18"/>
+      <c r="U5" s="18"/>
+      <c r="V5" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="W5" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="X5" s="13">
+        <f t="shared" si="0"/>
+        <v>59.12</v>
+      </c>
+      <c r="Y5" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="Z5" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AA5" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AB5" s="13">
+        <f t="shared" si="0"/>
+        <v>59.12</v>
+      </c>
+      <c r="AC5" s="13">
+        <f t="shared" si="0"/>
+        <v>328.47</v>
+      </c>
+      <c r="AD5" s="13">
+        <f t="shared" si="0"/>
+        <v>120</v>
+      </c>
+      <c r="AE5" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AF5" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AG5" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AH5" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AI5" s="13">
+        <f t="shared" si="0"/>
+        <v>328.47</v>
+      </c>
+      <c r="AJ5" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AK5" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AL5" s="23"/>
+      <c r="AM5" s="23"/>
+      <c r="AN5" s="23"/>
+      <c r="AO5" s="23"/>
+      <c r="AP5" s="23"/>
+      <c r="AQ5" s="23"/>
+      <c r="AR5" s="23"/>
+      <c r="AS5" s="9"/>
+      <c r="AT5" s="9"/>
+      <c r="AU5" s="30"/>
+      <c r="AV5" s="30"/>
+      <c r="AW5" s="9"/>
+      <c r="AX5" s="9"/>
+      <c r="AY5" s="9"/>
+      <c r="AZ5" s="9"/>
+      <c r="BA5" s="9"/>
+      <c r="BB5" s="9"/>
+      <c r="BC5" s="9"/>
+      <c r="BD5" s="9"/>
+      <c r="BE5" s="9"/>
+      <c r="BF5" s="9"/>
+      <c r="BG5" s="9"/>
+      <c r="BH5" s="9"/>
+      <c r="BI5" s="9"/>
+      <c r="BJ5" s="9"/>
+      <c r="BK5" s="9"/>
+      <c r="BL5" s="9"/>
+      <c r="BM5" s="9"/>
+      <c r="BN5" s="9"/>
+      <c r="BO5" s="9"/>
+      <c r="BP5" s="30"/>
+      <c r="BQ5" s="30"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:B2"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="AS4" r:id="rId1" display="INS WH-1" tooltip="https://webappqc.roadmaperp.com:8765/ords/r/rmqc27/scm-us9011/warehouse1?p367019101_rowid=AAATkUAAHAADnkPAAX&amp;p367019101_store_id=INS WH-1&amp;session=1523407412914"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>

</xml_diff>